<commit_message>
Update sample inventory data for Snipe-IT
</commit_message>
<xml_diff>
--- a/data/Dummy data.xlsx
+++ b/data/Dummy data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nadhifaazka/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nadhifaazka/Documents/Intern Privy/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{137DDD92-0268-E842-8CA2-6F5121AC5543}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C0BEC96-4928-FB4C-956F-1FB65A462A90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16340" xr2:uid="{E460BB3F-4FF0-1D4F-8F63-FB9F8008A7DA}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="116">
   <si>
     <t>Asset Tag</t>
   </si>
@@ -148,9 +148,6 @@
     <t>Dell</t>
   </si>
   <si>
-    <t>Deployed</t>
-  </si>
-  <si>
     <t xml:space="preserve">Jakarta </t>
   </si>
   <si>
@@ -166,27 +163,18 @@
     <t xml:space="preserve">Apple </t>
   </si>
   <si>
-    <t xml:space="preserve">Ready to Deployed </t>
-  </si>
-  <si>
     <t>DLL1111</t>
   </si>
   <si>
     <t>APP1122</t>
   </si>
   <si>
-    <t>Alma</t>
-  </si>
-  <si>
     <t>ThinkPad</t>
   </si>
   <si>
     <t>Lenovo</t>
   </si>
   <si>
-    <t>In Repair</t>
-  </si>
-  <si>
     <t>LNO1223</t>
   </si>
   <si>
@@ -253,9 +241,6 @@
     <t>Logitech</t>
   </si>
   <si>
-    <t>Archived</t>
-  </si>
-  <si>
     <t>LGT7566</t>
   </si>
   <si>
@@ -349,24 +334,15 @@
     <t>Juan</t>
   </si>
   <si>
-    <t>Alya</t>
-  </si>
-  <si>
     <t>Afi</t>
   </si>
   <si>
-    <t>Vino</t>
-  </si>
-  <si>
     <t>Nena</t>
   </si>
   <si>
     <t xml:space="preserve">Ayu </t>
   </si>
   <si>
-    <t>Andi</t>
-  </si>
-  <si>
     <t>Kina</t>
   </si>
   <si>
@@ -376,9 +352,6 @@
     <t>Yoga</t>
   </si>
   <si>
-    <t>Brian</t>
-  </si>
-  <si>
     <t>Salman</t>
   </si>
   <si>
@@ -388,13 +361,28 @@
     <t xml:space="preserve">Dimas </t>
   </si>
   <si>
-    <t>Didi</t>
-  </si>
-  <si>
-    <t>Kevin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kunta </t>
+    <t>Mac Address</t>
+  </si>
+  <si>
+    <t>CPU</t>
+  </si>
+  <si>
+    <t>RAM</t>
+  </si>
+  <si>
+    <t>Storage</t>
+  </si>
+  <si>
+    <t>Operating System</t>
+  </si>
+  <si>
+    <t>Graphics</t>
+  </si>
+  <si>
+    <t>Privy HQ</t>
+  </si>
+  <si>
+    <t>Privy Quarter</t>
   </si>
 </sst>
 </file>
@@ -438,12 +426,18 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -458,7 +452,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -466,6 +460,8 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -780,22 +776,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61CE36BB-B836-FE48-96B8-B2CA2E34C478}">
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:R25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.83203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -808,28 +810,46 @@
       <c r="D1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="8" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="6" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="K1" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="L1" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="M1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="N1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="O1" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="P1" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1"/>
-      <c r="L1" s="2"/>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="Q1" s="1"/>
+      <c r="R1" s="2"/>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -842,759 +862,735 @@
       <c r="D2" t="s">
         <v>36</v>
       </c>
-      <c r="E2" t="s">
-        <v>37</v>
+      <c r="E2">
+        <v>5</v>
       </c>
       <c r="F2" t="s">
-        <v>44</v>
-      </c>
-      <c r="G2" s="3">
+        <v>42</v>
+      </c>
+      <c r="M2" s="3">
         <v>45294</v>
       </c>
-      <c r="H2" s="4">
+      <c r="N2" s="4">
         <v>13000000</v>
       </c>
-      <c r="I2" t="s">
+      <c r="O2" t="s">
+        <v>114</v>
+      </c>
+      <c r="P2" t="s">
         <v>38</v>
       </c>
-      <c r="J2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="C3" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D3" t="s">
-        <v>60</v>
-      </c>
-      <c r="E3" t="s">
-        <v>43</v>
+        <v>56</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
       </c>
       <c r="F3" t="s">
-        <v>61</v>
-      </c>
-      <c r="G3" s="3">
+        <v>57</v>
+      </c>
+      <c r="M3" s="3">
         <v>45316</v>
       </c>
-      <c r="H3">
+      <c r="N3">
         <v>12000000</v>
       </c>
-      <c r="I3" t="s">
-        <v>95</v>
-      </c>
-      <c r="J3" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="O3" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C4" t="s">
         <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>48</v>
-      </c>
-      <c r="E4" t="s">
-        <v>49</v>
+        <v>45</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>50</v>
-      </c>
-      <c r="G4" s="3">
+        <v>46</v>
+      </c>
+      <c r="M4" s="3">
         <v>45325</v>
       </c>
-      <c r="H4">
+      <c r="N4">
         <v>19000000</v>
       </c>
-      <c r="I4" t="s">
-        <v>38</v>
-      </c>
-      <c r="J4" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="O4" t="s">
+        <v>37</v>
+      </c>
+      <c r="P4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C5" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D5" t="s">
-        <v>60</v>
-      </c>
-      <c r="E5" t="s">
-        <v>49</v>
+        <v>56</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>63</v>
-      </c>
-      <c r="G5" s="3">
+        <v>59</v>
+      </c>
+      <c r="M5" s="3">
         <v>45373</v>
       </c>
-      <c r="H5">
+      <c r="N5">
         <v>20000000</v>
       </c>
-      <c r="I5" t="s">
-        <v>38</v>
-      </c>
-      <c r="J5" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="O5" t="s">
+        <v>37</v>
+      </c>
+      <c r="P5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>14</v>
       </c>
       <c r="B6" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C6" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D6" t="s">
-        <v>42</v>
-      </c>
-      <c r="E6" t="s">
-        <v>37</v>
+        <v>41</v>
+      </c>
+      <c r="E6">
+        <v>5</v>
       </c>
       <c r="F6" t="s">
-        <v>66</v>
-      </c>
-      <c r="G6" s="3">
+        <v>62</v>
+      </c>
+      <c r="M6" s="3">
         <v>45399</v>
       </c>
-      <c r="H6">
+      <c r="N6">
         <v>16000000</v>
       </c>
-      <c r="I6" t="s">
-        <v>38</v>
-      </c>
-      <c r="J6" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="O6" t="s">
+        <v>37</v>
+      </c>
+      <c r="P6" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>15</v>
       </c>
       <c r="B7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" t="s">
         <v>40</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>41</v>
       </c>
-      <c r="D7" t="s">
-        <v>42</v>
-      </c>
-      <c r="E7" t="s">
+      <c r="E7">
+        <v>2</v>
+      </c>
+      <c r="F7" t="s">
         <v>43</v>
       </c>
-      <c r="F7" t="s">
-        <v>45</v>
-      </c>
-      <c r="G7" s="3">
+      <c r="M7" s="3">
         <v>45415</v>
       </c>
-      <c r="H7">
+      <c r="N7">
         <v>24000000</v>
       </c>
-      <c r="I7" t="s">
-        <v>38</v>
-      </c>
-      <c r="J7" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="O7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>16</v>
       </c>
       <c r="B8" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C8" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D8" t="s">
-        <v>42</v>
-      </c>
-      <c r="E8" t="s">
-        <v>43</v>
+        <v>41</v>
+      </c>
+      <c r="E8">
+        <v>2</v>
       </c>
       <c r="F8" t="s">
-        <v>67</v>
-      </c>
-      <c r="G8" s="3">
+        <v>63</v>
+      </c>
+      <c r="M8" s="3">
         <v>45427</v>
       </c>
-      <c r="H8">
+      <c r="N8">
         <v>16000000</v>
       </c>
-      <c r="I8" t="s">
-        <v>38</v>
-      </c>
-      <c r="J8" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="O8" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>17</v>
       </c>
       <c r="B9" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C9" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="D9" t="s">
-        <v>71</v>
-      </c>
-      <c r="E9" t="s">
-        <v>72</v>
+        <v>67</v>
+      </c>
+      <c r="E9">
+        <v>3</v>
       </c>
       <c r="F9" t="s">
-        <v>73</v>
-      </c>
-      <c r="G9" s="3">
+        <v>68</v>
+      </c>
+      <c r="M9" s="3">
         <v>45443</v>
       </c>
-      <c r="H9">
+      <c r="N9">
         <v>180000</v>
       </c>
-      <c r="I9" t="s">
-        <v>38</v>
-      </c>
-      <c r="J9" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="O9" t="s">
+        <v>37</v>
+      </c>
+      <c r="P9" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>18</v>
       </c>
       <c r="B10" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C10" t="s">
         <v>34</v>
       </c>
       <c r="D10" t="s">
-        <v>42</v>
-      </c>
-      <c r="E10" t="s">
-        <v>37</v>
+        <v>41</v>
+      </c>
+      <c r="E10">
+        <v>5</v>
       </c>
       <c r="F10" t="s">
-        <v>53</v>
-      </c>
-      <c r="G10" s="3">
+        <v>49</v>
+      </c>
+      <c r="M10" s="3">
         <v>45432</v>
       </c>
-      <c r="H10">
+      <c r="N10">
         <v>35000000</v>
       </c>
-      <c r="I10" t="s">
-        <v>38</v>
-      </c>
-      <c r="J10" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="O10" t="s">
+        <v>37</v>
+      </c>
+      <c r="P10" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>19</v>
       </c>
       <c r="B11" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="C11" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="D11" t="s">
-        <v>56</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>43</v>
+        <v>52</v>
+      </c>
+      <c r="E11" s="5">
+        <v>2</v>
       </c>
       <c r="F11" t="s">
-        <v>79</v>
-      </c>
-      <c r="G11" s="3">
+        <v>74</v>
+      </c>
+      <c r="M11" s="3">
         <v>45444</v>
       </c>
-      <c r="H11">
+      <c r="N11">
         <v>2900000</v>
       </c>
-      <c r="I11" t="s">
-        <v>38</v>
-      </c>
-      <c r="J11" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="O11" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>20</v>
       </c>
       <c r="B12" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="C12" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="D12" t="s">
-        <v>56</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>43</v>
+        <v>52</v>
+      </c>
+      <c r="E12" s="5">
+        <v>2</v>
       </c>
       <c r="F12" t="s">
-        <v>80</v>
-      </c>
-      <c r="G12" s="3">
+        <v>75</v>
+      </c>
+      <c r="M12" s="3">
         <v>45453</v>
       </c>
-      <c r="H12">
+      <c r="N12">
         <v>2900000</v>
       </c>
-      <c r="I12" t="s">
-        <v>38</v>
-      </c>
-      <c r="J12" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="O12" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>21</v>
       </c>
       <c r="B13" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C13" t="s">
         <v>34</v>
       </c>
       <c r="D13" t="s">
-        <v>56</v>
-      </c>
-      <c r="E13" t="s">
-        <v>37</v>
+        <v>52</v>
+      </c>
+      <c r="E13">
+        <v>5</v>
       </c>
       <c r="F13" t="s">
-        <v>57</v>
-      </c>
-      <c r="G13" s="3">
+        <v>53</v>
+      </c>
+      <c r="M13" s="3">
         <v>45455</v>
       </c>
-      <c r="H13">
+      <c r="N13">
         <v>21000000</v>
       </c>
-      <c r="I13" t="s">
-        <v>38</v>
-      </c>
-      <c r="J13" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="O13" t="s">
+        <v>37</v>
+      </c>
+      <c r="P13" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>22</v>
       </c>
       <c r="B14" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C14" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="D14" t="s">
-        <v>42</v>
-      </c>
-      <c r="E14" t="s">
-        <v>72</v>
+        <v>41</v>
+      </c>
+      <c r="E14">
+        <v>3</v>
       </c>
       <c r="F14" t="s">
-        <v>91</v>
-      </c>
-      <c r="G14" s="3">
+        <v>86</v>
+      </c>
+      <c r="M14" s="3">
         <v>45474</v>
       </c>
-      <c r="H14">
+      <c r="N14">
         <v>14000000</v>
       </c>
-      <c r="I14" t="s">
-        <v>38</v>
-      </c>
-      <c r="J14" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="O14" t="s">
+        <v>37</v>
+      </c>
+      <c r="P14" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>23</v>
       </c>
       <c r="B15" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="C15" t="s">
+        <v>73</v>
+      </c>
+      <c r="D15" t="s">
+        <v>45</v>
+      </c>
+      <c r="E15">
+        <v>5</v>
+      </c>
+      <c r="F15" t="s">
         <v>78</v>
       </c>
-      <c r="D15" t="s">
-        <v>48</v>
-      </c>
-      <c r="E15" t="s">
-        <v>37</v>
-      </c>
-      <c r="F15" t="s">
-        <v>83</v>
-      </c>
-      <c r="G15" s="3">
+      <c r="M15" s="3">
         <v>45483</v>
       </c>
-      <c r="H15">
+      <c r="N15">
         <v>6100000</v>
       </c>
-      <c r="I15" t="s">
-        <v>38</v>
-      </c>
-      <c r="J15" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="O15" t="s">
+        <v>37</v>
+      </c>
+      <c r="P15" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>24</v>
       </c>
       <c r="B16" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="C16" t="s">
+        <v>85</v>
+      </c>
+      <c r="D16" t="s">
+        <v>88</v>
+      </c>
+      <c r="E16">
+        <v>2</v>
+      </c>
+      <c r="F16" t="s">
+        <v>89</v>
+      </c>
+      <c r="M16" s="3">
+        <v>45514</v>
+      </c>
+      <c r="N16">
+        <v>11000000</v>
+      </c>
+      <c r="O16" t="s">
         <v>90</v>
       </c>
-      <c r="D16" t="s">
-        <v>93</v>
-      </c>
-      <c r="E16" t="s">
-        <v>43</v>
-      </c>
-      <c r="F16" t="s">
-        <v>94</v>
-      </c>
-      <c r="G16" s="3">
-        <v>45514</v>
-      </c>
-      <c r="H16">
-        <v>11000000</v>
-      </c>
-      <c r="I16" t="s">
-        <v>95</v>
-      </c>
-      <c r="J16" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>25</v>
       </c>
       <c r="B17" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C17" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="D17" t="s">
+        <v>67</v>
+      </c>
+      <c r="E17">
+        <v>5</v>
+      </c>
+      <c r="F17" t="s">
         <v>71</v>
       </c>
-      <c r="E17" t="s">
-        <v>37</v>
-      </c>
-      <c r="F17" t="s">
-        <v>76</v>
-      </c>
-      <c r="G17" s="3">
+      <c r="M17" s="3">
         <v>45563</v>
       </c>
-      <c r="H17">
+      <c r="N17">
         <v>180000</v>
       </c>
-      <c r="I17" t="s">
-        <v>38</v>
-      </c>
-      <c r="J17" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="O17" t="s">
+        <v>37</v>
+      </c>
+      <c r="P17" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>26</v>
       </c>
       <c r="B18" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="C18" t="s">
+        <v>92</v>
+      </c>
+      <c r="D18" t="s">
+        <v>93</v>
+      </c>
+      <c r="E18">
+        <v>5</v>
+      </c>
+      <c r="F18" t="s">
+        <v>94</v>
+      </c>
+      <c r="M18" s="3">
+        <v>45584</v>
+      </c>
+      <c r="N18">
+        <v>2250000</v>
+      </c>
+      <c r="O18" t="s">
+        <v>37</v>
+      </c>
+      <c r="P18" t="s">
         <v>97</v>
       </c>
-      <c r="D18" t="s">
-        <v>98</v>
-      </c>
-      <c r="E18" t="s">
-        <v>37</v>
-      </c>
-      <c r="F18" t="s">
-        <v>99</v>
-      </c>
-      <c r="G18" s="3">
-        <v>45584</v>
-      </c>
-      <c r="H18">
-        <v>2250000</v>
-      </c>
-      <c r="I18" t="s">
-        <v>38</v>
-      </c>
-      <c r="J18" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>27</v>
       </c>
       <c r="B19" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="C19" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D19" t="s">
+        <v>93</v>
+      </c>
+      <c r="E19">
+        <v>5</v>
+      </c>
+      <c r="F19" t="s">
+        <v>95</v>
+      </c>
+      <c r="M19" s="3">
+        <v>45593</v>
+      </c>
+      <c r="N19">
+        <v>2250000</v>
+      </c>
+      <c r="O19" t="s">
+        <v>37</v>
+      </c>
+      <c r="P19" t="s">
         <v>98</v>
       </c>
-      <c r="E19" t="s">
-        <v>37</v>
-      </c>
-      <c r="F19" t="s">
-        <v>100</v>
-      </c>
-      <c r="G19" s="3">
-        <v>45593</v>
-      </c>
-      <c r="H19">
-        <v>2250000</v>
-      </c>
-      <c r="I19" t="s">
-        <v>38</v>
-      </c>
-      <c r="J19" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>28</v>
       </c>
       <c r="B20" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="C20" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="D20" t="s">
-        <v>48</v>
-      </c>
-      <c r="E20" t="s">
-        <v>43</v>
+        <v>45</v>
+      </c>
+      <c r="E20">
+        <v>2</v>
       </c>
       <c r="F20" t="s">
-        <v>82</v>
-      </c>
-      <c r="G20" s="3">
+        <v>77</v>
+      </c>
+      <c r="M20" s="3">
         <v>45606</v>
       </c>
-      <c r="H20">
+      <c r="N20">
         <v>6100000</v>
       </c>
-      <c r="I20" t="s">
-        <v>38</v>
-      </c>
-      <c r="J20" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="O20" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>29</v>
       </c>
       <c r="B21" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C21" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D21" t="s">
-        <v>60</v>
-      </c>
-      <c r="E21" t="s">
-        <v>37</v>
+        <v>56</v>
+      </c>
+      <c r="E21">
+        <v>5</v>
       </c>
       <c r="F21" t="s">
-        <v>68</v>
-      </c>
-      <c r="G21" s="3">
+        <v>64</v>
+      </c>
+      <c r="M21" s="3">
         <v>45615</v>
       </c>
-      <c r="H21">
+      <c r="N21">
         <v>25000000</v>
       </c>
-      <c r="I21" t="s">
-        <v>38</v>
-      </c>
-      <c r="J21" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="O21" t="s">
+        <v>37</v>
+      </c>
+      <c r="P21" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>30</v>
       </c>
       <c r="B22" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="C22" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="D22" t="s">
         <v>36</v>
       </c>
-      <c r="E22" t="s">
-        <v>43</v>
+      <c r="E22">
+        <v>2</v>
       </c>
       <c r="F22" t="s">
-        <v>88</v>
-      </c>
-      <c r="G22" s="3">
+        <v>83</v>
+      </c>
+      <c r="M22" s="3">
         <v>45623</v>
       </c>
-      <c r="H22">
+      <c r="N22">
         <v>120000</v>
       </c>
-      <c r="I22" t="s">
-        <v>95</v>
-      </c>
-      <c r="J22" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="O22" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>31</v>
       </c>
       <c r="B23" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="C23" t="s">
+        <v>66</v>
+      </c>
+      <c r="D23" t="s">
+        <v>67</v>
+      </c>
+      <c r="E23">
+        <v>4</v>
+      </c>
+      <c r="F23" t="s">
         <v>70</v>
       </c>
-      <c r="D23" t="s">
-        <v>71</v>
-      </c>
-      <c r="E23" t="s">
-        <v>49</v>
-      </c>
-      <c r="F23" t="s">
-        <v>75</v>
-      </c>
-      <c r="G23" s="3">
+      <c r="M23" s="3">
         <v>45628</v>
       </c>
-      <c r="H23">
+      <c r="N23">
         <v>1800000</v>
       </c>
-      <c r="I23" t="s">
-        <v>38</v>
-      </c>
-      <c r="J23" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="O23" t="s">
+        <v>37</v>
+      </c>
+      <c r="P23" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>32</v>
       </c>
       <c r="B24" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="C24" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="D24" t="s">
-        <v>71</v>
-      </c>
-      <c r="E24" t="s">
-        <v>37</v>
+        <v>67</v>
+      </c>
+      <c r="E24">
+        <v>4</v>
       </c>
       <c r="F24" t="s">
-        <v>86</v>
-      </c>
-      <c r="G24" s="3">
+        <v>81</v>
+      </c>
+      <c r="M24" s="3">
         <v>45636</v>
       </c>
-      <c r="H24">
+      <c r="N24">
         <v>150000</v>
       </c>
-      <c r="I24" t="s">
-        <v>95</v>
-      </c>
-      <c r="J24" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="O24" t="s">
+        <v>90</v>
+      </c>
+      <c r="P24" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>33</v>
       </c>
       <c r="B25" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C25" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="D25" t="s">
+        <v>67</v>
+      </c>
+      <c r="E25">
+        <v>3</v>
+      </c>
+      <c r="F25" t="s">
         <v>71</v>
       </c>
-      <c r="E25" t="s">
-        <v>72</v>
-      </c>
-      <c r="F25" t="s">
-        <v>76</v>
-      </c>
-      <c r="G25" s="3">
+      <c r="M25" s="3">
         <v>45638</v>
       </c>
-      <c r="H25">
+      <c r="N25">
         <v>180000</v>
       </c>
-      <c r="I25" t="s">
-        <v>38</v>
-      </c>
-      <c r="J25" t="s">
-        <v>111</v>
+      <c r="O25" t="s">
+        <v>37</v>
+      </c>
+      <c r="P25" t="s">
+        <v>103</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update sample inventory data
</commit_message>
<xml_diff>
--- a/data/Dummy data.xlsx
+++ b/data/Dummy data.xlsx
@@ -5,16 +5,19 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nadhifaazka/Documents/Intern Privy/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nadhifaazka/Documents/GitHub/privy-snipeit/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C0BEC96-4928-FB4C-956F-1FB65A462A90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FA55334-3E10-8146-A774-4D81EBDEFAD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16340" xr2:uid="{E460BB3F-4FF0-1D4F-8F63-FB9F8008A7DA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$P$25</definedName>
+  </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -35,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="183">
   <si>
     <t>Asset Tag</t>
   </si>
@@ -148,9 +151,6 @@
     <t>Dell</t>
   </si>
   <si>
-    <t xml:space="preserve">Jakarta </t>
-  </si>
-  <si>
     <t>Sarah</t>
   </si>
   <si>
@@ -244,9 +244,6 @@
     <t>LGT7566</t>
   </si>
   <si>
-    <t>MX Key S</t>
-  </si>
-  <si>
     <t>LGT4421</t>
   </si>
   <si>
@@ -301,21 +298,9 @@
     <t>Veriton X</t>
   </si>
   <si>
-    <t>Asus</t>
-  </si>
-  <si>
-    <t>ASS1238</t>
-  </si>
-  <si>
-    <t>Jogja</t>
-  </si>
-  <si>
     <t>Microsoft 365 Business Standard</t>
   </si>
   <si>
-    <t>Mics Software</t>
-  </si>
-  <si>
     <t xml:space="preserve">Microsoft </t>
   </si>
   <si>
@@ -337,9 +322,6 @@
     <t>Afi</t>
   </si>
   <si>
-    <t>Nena</t>
-  </si>
-  <si>
     <t xml:space="preserve">Ayu </t>
   </si>
   <si>
@@ -349,9 +331,6 @@
     <t>Fajar</t>
   </si>
   <si>
-    <t>Yoga</t>
-  </si>
-  <si>
     <t>Salman</t>
   </si>
   <si>
@@ -383,6 +362,231 @@
   </si>
   <si>
     <t>Privy Quarter</t>
+  </si>
+  <si>
+    <t>3C:52:82:A1:B2:C1</t>
+  </si>
+  <si>
+    <t>48:21:0B:D4:E5:F1</t>
+  </si>
+  <si>
+    <t>A4:BB:6D:11:22:01</t>
+  </si>
+  <si>
+    <t>A4:BB:6D:11:22:02</t>
+  </si>
+  <si>
+    <t>7A:9B:1C:2D:3E:01</t>
+  </si>
+  <si>
+    <t>8C:1F:64:A2:B3:C1</t>
+  </si>
+  <si>
+    <t>8C:1F:64:A2:B3:C3</t>
+  </si>
+  <si>
+    <t>A8:7C:F5:D4:E5:F1</t>
+  </si>
+  <si>
+    <t>A8:7C:F5:D4:E5:F2</t>
+  </si>
+  <si>
+    <t>8C:1F:64:A2:B3:C2</t>
+  </si>
+  <si>
+    <t>Intel Core i5-1335U</t>
+  </si>
+  <si>
+    <t>Intel Core Ultra 5 125U</t>
+  </si>
+  <si>
+    <t>Apple M3</t>
+  </si>
+  <si>
+    <t>Apple M4 Pro</t>
+  </si>
+  <si>
+    <t>Intel Core Ultra 5 125H</t>
+  </si>
+  <si>
+    <t>16 GB</t>
+  </si>
+  <si>
+    <t>24 GB</t>
+  </si>
+  <si>
+    <t>1 TB SSD</t>
+  </si>
+  <si>
+    <t>512 GB SSD</t>
+  </si>
+  <si>
+    <t>Windows 11 Pro</t>
+  </si>
+  <si>
+    <t>macOS Sequoia</t>
+  </si>
+  <si>
+    <t>Snapdragon 8 Gen 3</t>
+  </si>
+  <si>
+    <t>Apple A16 Bionic</t>
+  </si>
+  <si>
+    <t>8 GB</t>
+  </si>
+  <si>
+    <t>12 GB</t>
+  </si>
+  <si>
+    <t>6 GB</t>
+  </si>
+  <si>
+    <t>256 GB</t>
+  </si>
+  <si>
+    <t>128 GB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">512 GB  </t>
+  </si>
+  <si>
+    <t>Android 15</t>
+  </si>
+  <si>
+    <t>iOS 18</t>
+  </si>
+  <si>
+    <t>Adreno 750</t>
+  </si>
+  <si>
+    <t>Apple GPU (5-core)</t>
+  </si>
+  <si>
+    <t>A4:BB:6D:33:44:01</t>
+  </si>
+  <si>
+    <t>D8:5D:E2:44:55:11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apple M4  </t>
+  </si>
+  <si>
+    <t>Intel Core i5-14400</t>
+  </si>
+  <si>
+    <t>Acer</t>
+  </si>
+  <si>
+    <t>ACR1238</t>
+  </si>
+  <si>
+    <t>Intel UHD Graphics 730</t>
+  </si>
+  <si>
+    <t>LGT78826</t>
+  </si>
+  <si>
+    <t>Misc Software</t>
+  </si>
+  <si>
+    <t>MX Keys S</t>
+  </si>
+  <si>
+    <t>10:AA:22:BB:33:01</t>
+  </si>
+  <si>
+    <t>20:BB:33:CC:44:02</t>
+  </si>
+  <si>
+    <t>20:BB:33:CC:44:03</t>
+  </si>
+  <si>
+    <t>30:CC:44:DD:55:04</t>
+  </si>
+  <si>
+    <t>10:AA:22:BB:33:05</t>
+  </si>
+  <si>
+    <t>30:CC:44:DD:55:06</t>
+  </si>
+  <si>
+    <t>40:DD:55:EE:66:07</t>
+  </si>
+  <si>
+    <t>10:AA:22:BB:33:08</t>
+  </si>
+  <si>
+    <t>40:DD:55:EE:66:09</t>
+  </si>
+  <si>
+    <t>10:AA:22:BB:33:10</t>
+  </si>
+  <si>
+    <t>Embedded Controller</t>
+  </si>
+  <si>
+    <t>Display Controller</t>
+  </si>
+  <si>
+    <t>Cloud Service</t>
+  </si>
+  <si>
+    <t>128 MB</t>
+  </si>
+  <si>
+    <t>512 MB</t>
+  </si>
+  <si>
+    <t>64 MB</t>
+  </si>
+  <si>
+    <t>256 MB</t>
+  </si>
+  <si>
+    <t>32 MB</t>
+  </si>
+  <si>
+    <t>100 GB</t>
+  </si>
+  <si>
+    <t>16 MB</t>
+  </si>
+  <si>
+    <t>Firmware v1.10</t>
+  </si>
+  <si>
+    <t>Monitor Firmware</t>
+  </si>
+  <si>
+    <t>Microsoft 365</t>
+  </si>
+  <si>
+    <t>Firmware v2.10</t>
+  </si>
+  <si>
+    <t>Integrated</t>
+  </si>
+  <si>
+    <t>Virtual</t>
+  </si>
+  <si>
+    <t>A6:CC:29:12:22:07</t>
+  </si>
+  <si>
+    <t>A6:CC:29:12:22:10</t>
+  </si>
+  <si>
+    <t>Intel Iris Xe Graphics</t>
+  </si>
+  <si>
+    <t>Intel Iris Graphics</t>
+  </si>
+  <si>
+    <t>Apple Integrated GPU</t>
+  </si>
+  <si>
+    <t>Desktop</t>
   </si>
 </sst>
 </file>
@@ -426,18 +630,12 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -452,7 +650,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -460,7 +658,6 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -785,15 +982,15 @@
     <col min="4" max="4" width="12.83203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="6.83203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="5.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.83203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.83203125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="17.5" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.1640625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="14" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.83203125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="12.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -810,29 +1007,29 @@
       <c r="D1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="6" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="L1" s="6" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="M1" s="6" t="s">
         <v>6</v>
@@ -866,7 +1063,25 @@
         <v>5</v>
       </c>
       <c r="F2" t="s">
-        <v>42</v>
+        <v>41</v>
+      </c>
+      <c r="G2" t="s">
+        <v>108</v>
+      </c>
+      <c r="H2" t="s">
+        <v>118</v>
+      </c>
+      <c r="I2" t="s">
+        <v>123</v>
+      </c>
+      <c r="J2" t="s">
+        <v>126</v>
+      </c>
+      <c r="K2" t="s">
+        <v>127</v>
+      </c>
+      <c r="L2" t="s">
+        <v>179</v>
       </c>
       <c r="M2" s="3">
         <v>45294</v>
@@ -875,10 +1090,10 @@
         <v>13000000</v>
       </c>
       <c r="O2" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="P2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.2">
@@ -886,19 +1101,37 @@
         <v>11</v>
       </c>
       <c r="B3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D3" t="s">
         <v>55</v>
-      </c>
-      <c r="C3" t="s">
-        <v>61</v>
-      </c>
-      <c r="D3" t="s">
-        <v>56</v>
       </c>
       <c r="E3">
         <v>2</v>
       </c>
       <c r="F3" t="s">
-        <v>57</v>
+        <v>56</v>
+      </c>
+      <c r="G3" t="s">
+        <v>113</v>
+      </c>
+      <c r="H3" t="s">
+        <v>129</v>
+      </c>
+      <c r="I3" t="s">
+        <v>131</v>
+      </c>
+      <c r="J3" t="s">
+        <v>134</v>
+      </c>
+      <c r="K3" t="s">
+        <v>137</v>
+      </c>
+      <c r="L3" t="s">
+        <v>139</v>
       </c>
       <c r="M3" s="3">
         <v>45316</v>
@@ -907,7 +1140,7 @@
         <v>12000000</v>
       </c>
       <c r="O3" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.2">
@@ -915,19 +1148,37 @@
         <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C4" t="s">
         <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E4">
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>46</v>
+        <v>45</v>
+      </c>
+      <c r="G4" t="s">
+        <v>109</v>
+      </c>
+      <c r="H4" t="s">
+        <v>119</v>
+      </c>
+      <c r="I4" t="s">
+        <v>123</v>
+      </c>
+      <c r="J4" t="s">
+        <v>126</v>
+      </c>
+      <c r="K4" t="s">
+        <v>127</v>
+      </c>
+      <c r="L4" t="s">
+        <v>180</v>
       </c>
       <c r="M4" s="3">
         <v>45325</v>
@@ -936,10 +1187,10 @@
         <v>19000000</v>
       </c>
       <c r="O4" t="s">
-        <v>37</v>
+        <v>107</v>
       </c>
       <c r="P4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.2">
@@ -947,19 +1198,37 @@
         <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E5">
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>59</v>
+        <v>58</v>
+      </c>
+      <c r="G5" t="s">
+        <v>117</v>
+      </c>
+      <c r="H5" t="s">
+        <v>129</v>
+      </c>
+      <c r="I5" t="s">
+        <v>132</v>
+      </c>
+      <c r="J5" t="s">
+        <v>126</v>
+      </c>
+      <c r="K5" t="s">
+        <v>137</v>
+      </c>
+      <c r="L5" t="s">
+        <v>139</v>
       </c>
       <c r="M5" s="3">
         <v>45373</v>
@@ -968,10 +1237,10 @@
         <v>20000000</v>
       </c>
       <c r="O5" t="s">
-        <v>37</v>
+        <v>107</v>
       </c>
       <c r="P5" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.2">
@@ -979,19 +1248,37 @@
         <v>14</v>
       </c>
       <c r="B6" t="s">
+        <v>59</v>
+      </c>
+      <c r="C6" t="s">
         <v>60</v>
       </c>
-      <c r="C6" t="s">
-        <v>61</v>
-      </c>
       <c r="D6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E6">
         <v>5</v>
       </c>
       <c r="F6" t="s">
-        <v>62</v>
+        <v>61</v>
+      </c>
+      <c r="G6" t="s">
+        <v>115</v>
+      </c>
+      <c r="H6" t="s">
+        <v>130</v>
+      </c>
+      <c r="I6" t="s">
+        <v>133</v>
+      </c>
+      <c r="J6" t="s">
+        <v>134</v>
+      </c>
+      <c r="K6" t="s">
+        <v>138</v>
+      </c>
+      <c r="L6" t="s">
+        <v>140</v>
       </c>
       <c r="M6" s="3">
         <v>45399</v>
@@ -1000,10 +1287,10 @@
         <v>16000000</v>
       </c>
       <c r="O6" t="s">
-        <v>37</v>
+        <v>106</v>
       </c>
       <c r="P6" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.2">
@@ -1011,19 +1298,37 @@
         <v>15</v>
       </c>
       <c r="B7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C7" t="s">
         <v>39</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>40</v>
-      </c>
-      <c r="D7" t="s">
-        <v>41</v>
       </c>
       <c r="E7">
         <v>2</v>
       </c>
       <c r="F7" t="s">
-        <v>43</v>
+        <v>42</v>
+      </c>
+      <c r="G7" t="s">
+        <v>110</v>
+      </c>
+      <c r="H7" t="s">
+        <v>120</v>
+      </c>
+      <c r="I7" t="s">
+        <v>123</v>
+      </c>
+      <c r="J7" t="s">
+        <v>126</v>
+      </c>
+      <c r="K7" t="s">
+        <v>128</v>
+      </c>
+      <c r="L7" t="s">
+        <v>181</v>
       </c>
       <c r="M7" s="3">
         <v>45415</v>
@@ -1032,7 +1337,7 @@
         <v>24000000</v>
       </c>
       <c r="O7" t="s">
-        <v>37</v>
+        <v>107</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.2">
@@ -1040,19 +1345,37 @@
         <v>16</v>
       </c>
       <c r="B8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C8" t="s">
         <v>60</v>
       </c>
-      <c r="C8" t="s">
-        <v>61</v>
-      </c>
       <c r="D8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E8">
         <v>2</v>
       </c>
       <c r="F8" t="s">
-        <v>63</v>
+        <v>62</v>
+      </c>
+      <c r="G8" t="s">
+        <v>116</v>
+      </c>
+      <c r="H8" t="s">
+        <v>130</v>
+      </c>
+      <c r="I8" t="s">
+        <v>133</v>
+      </c>
+      <c r="J8" t="s">
+        <v>135</v>
+      </c>
+      <c r="K8" t="s">
+        <v>138</v>
+      </c>
+      <c r="L8" t="s">
+        <v>140</v>
       </c>
       <c r="M8" s="3">
         <v>45427</v>
@@ -1061,7 +1384,7 @@
         <v>16000000</v>
       </c>
       <c r="O8" t="s">
-        <v>37</v>
+        <v>107</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.2">
@@ -1069,19 +1392,37 @@
         <v>17</v>
       </c>
       <c r="B9" t="s">
+        <v>64</v>
+      </c>
+      <c r="C9" t="s">
         <v>65</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>66</v>
-      </c>
-      <c r="D9" t="s">
-        <v>67</v>
       </c>
       <c r="E9">
         <v>3</v>
       </c>
       <c r="F9" t="s">
-        <v>68</v>
+        <v>67</v>
+      </c>
+      <c r="G9" t="s">
+        <v>151</v>
+      </c>
+      <c r="H9" t="s">
+        <v>161</v>
+      </c>
+      <c r="I9" t="s">
+        <v>164</v>
+      </c>
+      <c r="J9" t="s">
+        <v>168</v>
+      </c>
+      <c r="K9" t="s">
+        <v>171</v>
+      </c>
+      <c r="L9" t="s">
+        <v>175</v>
       </c>
       <c r="M9" s="3">
         <v>45443</v>
@@ -1090,10 +1431,10 @@
         <v>180000</v>
       </c>
       <c r="O9" t="s">
-        <v>37</v>
+        <v>106</v>
       </c>
       <c r="P9" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.2">
@@ -1101,19 +1442,37 @@
         <v>18</v>
       </c>
       <c r="B10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C10" t="s">
         <v>34</v>
       </c>
       <c r="D10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E10">
         <v>5</v>
       </c>
       <c r="F10" t="s">
-        <v>49</v>
+        <v>48</v>
+      </c>
+      <c r="G10" t="s">
+        <v>111</v>
+      </c>
+      <c r="H10" t="s">
+        <v>121</v>
+      </c>
+      <c r="I10" t="s">
+        <v>124</v>
+      </c>
+      <c r="J10" t="s">
+        <v>125</v>
+      </c>
+      <c r="K10" t="s">
+        <v>128</v>
+      </c>
+      <c r="L10" t="s">
+        <v>181</v>
       </c>
       <c r="M10" s="3">
         <v>45432</v>
@@ -1122,10 +1481,10 @@
         <v>35000000</v>
       </c>
       <c r="O10" t="s">
-        <v>37</v>
+        <v>106</v>
       </c>
       <c r="P10" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.2">
@@ -1133,19 +1492,37 @@
         <v>19</v>
       </c>
       <c r="B11" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C11" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D11" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E11" s="5">
         <v>2</v>
       </c>
       <c r="F11" t="s">
-        <v>74</v>
+        <v>72</v>
+      </c>
+      <c r="G11" t="s">
+        <v>152</v>
+      </c>
+      <c r="H11" t="s">
+        <v>162</v>
+      </c>
+      <c r="I11" t="s">
+        <v>165</v>
+      </c>
+      <c r="J11" t="s">
+        <v>164</v>
+      </c>
+      <c r="K11" t="s">
+        <v>172</v>
+      </c>
+      <c r="L11" t="s">
+        <v>175</v>
       </c>
       <c r="M11" s="3">
         <v>45444</v>
@@ -1154,7 +1531,7 @@
         <v>2900000</v>
       </c>
       <c r="O11" t="s">
-        <v>37</v>
+        <v>107</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.2">
@@ -1162,19 +1539,37 @@
         <v>20</v>
       </c>
       <c r="B12" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C12" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D12" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E12" s="5">
         <v>2</v>
       </c>
       <c r="F12" t="s">
-        <v>75</v>
+        <v>73</v>
+      </c>
+      <c r="G12" t="s">
+        <v>153</v>
+      </c>
+      <c r="H12" t="s">
+        <v>162</v>
+      </c>
+      <c r="I12" t="s">
+        <v>165</v>
+      </c>
+      <c r="J12" t="s">
+        <v>164</v>
+      </c>
+      <c r="K12" t="s">
+        <v>172</v>
+      </c>
+      <c r="L12" t="s">
+        <v>175</v>
       </c>
       <c r="M12" s="3">
         <v>45453</v>
@@ -1183,7 +1578,7 @@
         <v>2900000</v>
       </c>
       <c r="O12" t="s">
-        <v>37</v>
+        <v>107</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.2">
@@ -1191,19 +1586,37 @@
         <v>21</v>
       </c>
       <c r="B13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C13" t="s">
         <v>34</v>
       </c>
       <c r="D13" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E13">
         <v>5</v>
       </c>
       <c r="F13" t="s">
-        <v>53</v>
+        <v>52</v>
+      </c>
+      <c r="G13" t="s">
+        <v>112</v>
+      </c>
+      <c r="H13" t="s">
+        <v>122</v>
+      </c>
+      <c r="I13" t="s">
+        <v>123</v>
+      </c>
+      <c r="J13" t="s">
+        <v>126</v>
+      </c>
+      <c r="K13" t="s">
+        <v>127</v>
+      </c>
+      <c r="L13" t="s">
+        <v>181</v>
       </c>
       <c r="M13" s="3">
         <v>45455</v>
@@ -1212,10 +1625,10 @@
         <v>21000000</v>
       </c>
       <c r="O13" t="s">
-        <v>37</v>
+        <v>106</v>
       </c>
       <c r="P13" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.2">
@@ -1223,19 +1636,37 @@
         <v>22</v>
       </c>
       <c r="B14" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C14" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E14">
         <v>3</v>
       </c>
       <c r="F14" t="s">
-        <v>86</v>
+        <v>84</v>
+      </c>
+      <c r="G14" t="s">
+        <v>141</v>
+      </c>
+      <c r="H14" t="s">
+        <v>143</v>
+      </c>
+      <c r="I14" t="s">
+        <v>123</v>
+      </c>
+      <c r="J14" t="s">
+        <v>136</v>
+      </c>
+      <c r="K14" t="s">
+        <v>128</v>
+      </c>
+      <c r="L14" t="s">
+        <v>181</v>
       </c>
       <c r="M14" s="3">
         <v>45474</v>
@@ -1244,10 +1675,10 @@
         <v>14000000</v>
       </c>
       <c r="O14" t="s">
-        <v>37</v>
+        <v>107</v>
       </c>
       <c r="P14" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.2">
@@ -1255,19 +1686,37 @@
         <v>23</v>
       </c>
       <c r="B15" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E15">
         <v>5</v>
       </c>
       <c r="F15" t="s">
-        <v>78</v>
+        <v>76</v>
+      </c>
+      <c r="G15" t="s">
+        <v>154</v>
+      </c>
+      <c r="H15" t="s">
+        <v>162</v>
+      </c>
+      <c r="I15" t="s">
+        <v>165</v>
+      </c>
+      <c r="J15" t="s">
+        <v>164</v>
+      </c>
+      <c r="K15" t="s">
+        <v>172</v>
+      </c>
+      <c r="L15" t="s">
+        <v>175</v>
       </c>
       <c r="M15" s="3">
         <v>45483</v>
@@ -1275,11 +1724,11 @@
       <c r="N15">
         <v>6100000</v>
       </c>
-      <c r="O15" t="s">
-        <v>37</v>
+      <c r="O15" s="5" t="s">
+        <v>106</v>
       </c>
       <c r="P15" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.2">
@@ -1287,19 +1736,37 @@
         <v>24</v>
       </c>
       <c r="B16" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C16" t="s">
-        <v>85</v>
+        <v>182</v>
       </c>
       <c r="D16" t="s">
-        <v>88</v>
+        <v>145</v>
       </c>
       <c r="E16">
         <v>2</v>
       </c>
       <c r="F16" t="s">
-        <v>89</v>
+        <v>146</v>
+      </c>
+      <c r="G16" t="s">
+        <v>142</v>
+      </c>
+      <c r="H16" t="s">
+        <v>144</v>
+      </c>
+      <c r="I16" t="s">
+        <v>123</v>
+      </c>
+      <c r="J16" t="s">
+        <v>136</v>
+      </c>
+      <c r="K16" t="s">
+        <v>127</v>
+      </c>
+      <c r="L16" t="s">
+        <v>147</v>
       </c>
       <c r="M16" s="3">
         <v>45514</v>
@@ -1308,7 +1775,7 @@
         <v>11000000</v>
       </c>
       <c r="O16" t="s">
-        <v>90</v>
+        <v>107</v>
       </c>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.2">
@@ -1316,19 +1783,37 @@
         <v>25</v>
       </c>
       <c r="B17" t="s">
+        <v>64</v>
+      </c>
+      <c r="C17" t="s">
         <v>65</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
         <v>66</v>
-      </c>
-      <c r="D17" t="s">
-        <v>67</v>
       </c>
       <c r="E17">
         <v>5</v>
       </c>
       <c r="F17" t="s">
-        <v>71</v>
+        <v>148</v>
+      </c>
+      <c r="G17" t="s">
+        <v>155</v>
+      </c>
+      <c r="H17" t="s">
+        <v>161</v>
+      </c>
+      <c r="I17" t="s">
+        <v>164</v>
+      </c>
+      <c r="J17" t="s">
+        <v>168</v>
+      </c>
+      <c r="K17" t="s">
+        <v>171</v>
+      </c>
+      <c r="L17" t="s">
+        <v>175</v>
       </c>
       <c r="M17" s="3">
         <v>45563</v>
@@ -1336,11 +1821,11 @@
       <c r="N17">
         <v>180000</v>
       </c>
-      <c r="O17" t="s">
-        <v>37</v>
+      <c r="O17" s="5" t="s">
+        <v>106</v>
       </c>
       <c r="P17" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.2">
@@ -1348,19 +1833,37 @@
         <v>26</v>
       </c>
       <c r="B18" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="C18" t="s">
-        <v>92</v>
+        <v>149</v>
       </c>
       <c r="D18" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="E18">
         <v>5</v>
       </c>
       <c r="F18" t="s">
-        <v>94</v>
+        <v>88</v>
+      </c>
+      <c r="G18" t="s">
+        <v>177</v>
+      </c>
+      <c r="H18" t="s">
+        <v>163</v>
+      </c>
+      <c r="I18" t="s">
+        <v>131</v>
+      </c>
+      <c r="J18" t="s">
+        <v>169</v>
+      </c>
+      <c r="K18" t="s">
+        <v>173</v>
+      </c>
+      <c r="L18" t="s">
+        <v>176</v>
       </c>
       <c r="M18" s="3">
         <v>45584</v>
@@ -1369,10 +1872,10 @@
         <v>2250000</v>
       </c>
       <c r="O18" t="s">
-        <v>37</v>
+        <v>107</v>
       </c>
       <c r="P18" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.2">
@@ -1380,19 +1883,37 @@
         <v>27</v>
       </c>
       <c r="B19" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="C19" t="s">
-        <v>92</v>
+        <v>149</v>
       </c>
       <c r="D19" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="E19">
         <v>5</v>
       </c>
       <c r="F19" t="s">
-        <v>95</v>
+        <v>89</v>
+      </c>
+      <c r="G19" t="s">
+        <v>178</v>
+      </c>
+      <c r="H19" t="s">
+        <v>163</v>
+      </c>
+      <c r="I19" t="s">
+        <v>131</v>
+      </c>
+      <c r="J19" t="s">
+        <v>169</v>
+      </c>
+      <c r="K19" t="s">
+        <v>173</v>
+      </c>
+      <c r="L19" t="s">
+        <v>176</v>
       </c>
       <c r="M19" s="3">
         <v>45593</v>
@@ -1400,11 +1921,11 @@
       <c r="N19">
         <v>2250000</v>
       </c>
-      <c r="O19" t="s">
-        <v>37</v>
+      <c r="O19" s="5" t="s">
+        <v>106</v>
       </c>
       <c r="P19" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.2">
@@ -1412,19 +1933,37 @@
         <v>28</v>
       </c>
       <c r="B20" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C20" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D20" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E20">
         <v>2</v>
       </c>
       <c r="F20" t="s">
-        <v>77</v>
+        <v>75</v>
+      </c>
+      <c r="G20" t="s">
+        <v>156</v>
+      </c>
+      <c r="H20" t="s">
+        <v>162</v>
+      </c>
+      <c r="I20" t="s">
+        <v>165</v>
+      </c>
+      <c r="J20" t="s">
+        <v>164</v>
+      </c>
+      <c r="K20" t="s">
+        <v>172</v>
+      </c>
+      <c r="L20" t="s">
+        <v>175</v>
       </c>
       <c r="M20" s="3">
         <v>45606</v>
@@ -1432,8 +1971,8 @@
       <c r="N20">
         <v>6100000</v>
       </c>
-      <c r="O20" t="s">
-        <v>37</v>
+      <c r="O20" s="5" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.2">
@@ -1441,19 +1980,37 @@
         <v>29</v>
       </c>
       <c r="B21" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C21" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D21" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E21">
         <v>5</v>
       </c>
       <c r="F21" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+      <c r="G21" t="s">
+        <v>114</v>
+      </c>
+      <c r="H21" t="s">
+        <v>129</v>
+      </c>
+      <c r="I21" t="s">
+        <v>132</v>
+      </c>
+      <c r="J21" t="s">
+        <v>136</v>
+      </c>
+      <c r="K21" t="s">
+        <v>137</v>
+      </c>
+      <c r="L21" t="s">
+        <v>139</v>
       </c>
       <c r="M21" s="3">
         <v>45615</v>
@@ -1461,11 +2018,11 @@
       <c r="N21">
         <v>25000000</v>
       </c>
-      <c r="O21" t="s">
-        <v>37</v>
+      <c r="O21" s="5" t="s">
+        <v>106</v>
       </c>
       <c r="P21" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.2">
@@ -1473,10 +2030,10 @@
         <v>30</v>
       </c>
       <c r="B22" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C22" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D22" t="s">
         <v>36</v>
@@ -1485,7 +2042,25 @@
         <v>2</v>
       </c>
       <c r="F22" t="s">
-        <v>83</v>
+        <v>81</v>
+      </c>
+      <c r="G22" t="s">
+        <v>157</v>
+      </c>
+      <c r="H22" t="s">
+        <v>161</v>
+      </c>
+      <c r="I22" t="s">
+        <v>166</v>
+      </c>
+      <c r="J22" t="s">
+        <v>170</v>
+      </c>
+      <c r="K22" t="s">
+        <v>171</v>
+      </c>
+      <c r="L22" t="s">
+        <v>175</v>
       </c>
       <c r="M22" s="3">
         <v>45623</v>
@@ -1494,7 +2069,7 @@
         <v>120000</v>
       </c>
       <c r="O22" t="s">
-        <v>90</v>
+        <v>107</v>
       </c>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.2">
@@ -1502,19 +2077,37 @@
         <v>31</v>
       </c>
       <c r="B23" t="s">
-        <v>69</v>
+        <v>150</v>
       </c>
       <c r="C23" t="s">
+        <v>65</v>
+      </c>
+      <c r="D23" t="s">
         <v>66</v>
-      </c>
-      <c r="D23" t="s">
-        <v>67</v>
       </c>
       <c r="E23">
         <v>4</v>
       </c>
       <c r="F23" t="s">
-        <v>70</v>
+        <v>68</v>
+      </c>
+      <c r="G23" t="s">
+        <v>158</v>
+      </c>
+      <c r="H23" t="s">
+        <v>161</v>
+      </c>
+      <c r="I23" t="s">
+        <v>167</v>
+      </c>
+      <c r="J23" t="s">
+        <v>166</v>
+      </c>
+      <c r="K23" t="s">
+        <v>171</v>
+      </c>
+      <c r="L23" t="s">
+        <v>175</v>
       </c>
       <c r="M23" s="3">
         <v>45628</v>
@@ -1522,11 +2115,8 @@
       <c r="N23">
         <v>1800000</v>
       </c>
-      <c r="O23" t="s">
-        <v>37</v>
-      </c>
-      <c r="P23" t="s">
-        <v>100</v>
+      <c r="O23" s="5" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.2">
@@ -1534,19 +2124,37 @@
         <v>32</v>
       </c>
       <c r="B24" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C24" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D24" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E24">
         <v>4</v>
       </c>
       <c r="F24" t="s">
-        <v>81</v>
+        <v>79</v>
+      </c>
+      <c r="G24" t="s">
+        <v>159</v>
+      </c>
+      <c r="H24" t="s">
+        <v>161</v>
+      </c>
+      <c r="I24" t="s">
+        <v>166</v>
+      </c>
+      <c r="J24" t="s">
+        <v>170</v>
+      </c>
+      <c r="K24" t="s">
+        <v>174</v>
+      </c>
+      <c r="L24" t="s">
+        <v>175</v>
       </c>
       <c r="M24" s="3">
         <v>45636</v>
@@ -1554,11 +2162,8 @@
       <c r="N24">
         <v>150000</v>
       </c>
-      <c r="O24" t="s">
-        <v>90</v>
-      </c>
-      <c r="P24" t="s">
-        <v>104</v>
+      <c r="O24" s="5" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.2">
@@ -1566,19 +2171,37 @@
         <v>33</v>
       </c>
       <c r="B25" t="s">
+        <v>64</v>
+      </c>
+      <c r="C25" t="s">
         <v>65</v>
       </c>
-      <c r="C25" t="s">
+      <c r="D25" t="s">
         <v>66</v>
-      </c>
-      <c r="D25" t="s">
-        <v>67</v>
       </c>
       <c r="E25">
         <v>3</v>
       </c>
       <c r="F25" t="s">
-        <v>71</v>
+        <v>69</v>
+      </c>
+      <c r="G25" t="s">
+        <v>160</v>
+      </c>
+      <c r="H25" t="s">
+        <v>161</v>
+      </c>
+      <c r="I25" t="s">
+        <v>164</v>
+      </c>
+      <c r="J25" t="s">
+        <v>168</v>
+      </c>
+      <c r="K25" t="s">
+        <v>171</v>
+      </c>
+      <c r="L25" t="s">
+        <v>175</v>
       </c>
       <c r="M25" s="3">
         <v>45638</v>
@@ -1587,13 +2210,14 @@
         <v>180000</v>
       </c>
       <c r="O25" t="s">
-        <v>37</v>
+        <v>107</v>
       </c>
       <c r="P25" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:P25" xr:uid="{61CE36BB-B836-FE48-96B8-B2CA2E34C478}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated Dummy Data spelling
</commit_message>
<xml_diff>
--- a/data/Dummy data.xlsx
+++ b/data/Dummy data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11028"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nadhifaazka/Documents/GitHub/privy-snipeit/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xav/Documents/GitHub/privy-snipeit/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FA55334-3E10-8146-A774-4D81EBDEFAD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DB5F775-EFB5-A346-940D-F023E0A92EDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16340" xr2:uid="{E460BB3F-4FF0-1D4F-8F63-FB9F8008A7DA}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="28800" windowHeight="16340" xr2:uid="{E460BB3F-4FF0-1D4F-8F63-FB9F8008A7DA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -145,18 +145,12 @@
     <t>Laptop</t>
   </si>
   <si>
-    <t>Latitude</t>
-  </si>
-  <si>
     <t>Dell</t>
   </si>
   <si>
     <t>Sarah</t>
   </si>
   <si>
-    <t>Macbook Air M3</t>
-  </si>
-  <si>
     <t xml:space="preserve">Laptop </t>
   </si>
   <si>
@@ -181,9 +175,6 @@
     <t>Yaya</t>
   </si>
   <si>
-    <t>Macbook Pro 14 M4</t>
-  </si>
-  <si>
     <t>APP1213</t>
   </si>
   <si>
@@ -217,9 +208,6 @@
     <t>SMS2112</t>
   </si>
   <si>
-    <t>Iphone 15</t>
-  </si>
-  <si>
     <t>Phone</t>
   </si>
   <si>
@@ -286,9 +274,6 @@
     <t>DLL3445</t>
   </si>
   <si>
-    <t>Mac Mini M4</t>
-  </si>
-  <si>
     <t xml:space="preserve">Desktop </t>
   </si>
   <si>
@@ -587,6 +572,21 @@
   </si>
   <si>
     <t>Desktop</t>
+  </si>
+  <si>
+    <t>Latitude 5440</t>
+  </si>
+  <si>
+    <t>iPhone 15</t>
+  </si>
+  <si>
+    <t>Macbook Pro</t>
+  </si>
+  <si>
+    <t>Macbook Air</t>
+  </si>
+  <si>
+    <t>Mac Mini</t>
   </si>
 </sst>
 </file>
@@ -650,7 +650,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -658,7 +658,6 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -677,9 +676,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -717,7 +716,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -823,7 +822,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -965,7 +964,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1014,22 +1013,22 @@
         <v>5</v>
       </c>
       <c r="G1" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="K1" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="L1" s="6" t="s">
         <v>100</v>
-      </c>
-      <c r="H1" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="I1" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="J1" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="K1" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="L1" s="6" t="s">
-        <v>105</v>
       </c>
       <c r="M1" s="6" t="s">
         <v>6</v>
@@ -1037,7 +1036,7 @@
       <c r="N1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="O1" s="7" t="s">
+      <c r="O1" s="6" t="s">
         <v>8</v>
       </c>
       <c r="P1" s="6" t="s">
@@ -1051,37 +1050,37 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
+        <v>178</v>
       </c>
       <c r="C2" t="s">
         <v>34</v>
       </c>
       <c r="D2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E2">
         <v>5</v>
       </c>
       <c r="F2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G2" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="H2" t="s">
+        <v>113</v>
+      </c>
+      <c r="I2" t="s">
         <v>118</v>
       </c>
-      <c r="I2" t="s">
-        <v>123</v>
-      </c>
       <c r="J2" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="K2" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="L2" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="M2" s="3">
         <v>45294</v>
@@ -1090,10 +1089,10 @@
         <v>13000000</v>
       </c>
       <c r="O2" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="P2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.2">
@@ -1101,37 +1100,37 @@
         <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D3" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="E3">
         <v>2</v>
       </c>
       <c r="F3" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="G3" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="H3" t="s">
+        <v>124</v>
+      </c>
+      <c r="I3" t="s">
+        <v>126</v>
+      </c>
+      <c r="J3" t="s">
         <v>129</v>
       </c>
-      <c r="I3" t="s">
-        <v>131</v>
-      </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
+        <v>132</v>
+      </c>
+      <c r="L3" t="s">
         <v>134</v>
-      </c>
-      <c r="K3" t="s">
-        <v>137</v>
-      </c>
-      <c r="L3" t="s">
-        <v>139</v>
       </c>
       <c r="M3" s="3">
         <v>45316</v>
@@ -1140,7 +1139,7 @@
         <v>12000000</v>
       </c>
       <c r="O3" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.2">
@@ -1148,37 +1147,37 @@
         <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C4" t="s">
         <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E4">
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G4" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="H4" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="I4" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="J4" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="K4" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="L4" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="M4" s="3">
         <v>45325</v>
@@ -1187,10 +1186,10 @@
         <v>19000000</v>
       </c>
       <c r="O4" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="P4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.2">
@@ -1198,37 +1197,37 @@
         <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C5" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D5" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="E5">
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G5" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="H5" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="I5" t="s">
+        <v>127</v>
+      </c>
+      <c r="J5" t="s">
+        <v>121</v>
+      </c>
+      <c r="K5" t="s">
         <v>132</v>
       </c>
-      <c r="J5" t="s">
-        <v>126</v>
-      </c>
-      <c r="K5" t="s">
-        <v>137</v>
-      </c>
       <c r="L5" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="M5" s="3">
         <v>45373</v>
@@ -1237,10 +1236,10 @@
         <v>20000000</v>
       </c>
       <c r="O5" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="P5" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.2">
@@ -1248,37 +1247,37 @@
         <v>14</v>
       </c>
       <c r="B6" t="s">
-        <v>59</v>
+        <v>179</v>
       </c>
       <c r="C6" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D6" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E6">
         <v>5</v>
       </c>
       <c r="F6" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="G6" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="H6" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="I6" t="s">
+        <v>128</v>
+      </c>
+      <c r="J6" t="s">
+        <v>129</v>
+      </c>
+      <c r="K6" t="s">
         <v>133</v>
       </c>
-      <c r="J6" t="s">
-        <v>134</v>
-      </c>
-      <c r="K6" t="s">
-        <v>138</v>
-      </c>
       <c r="L6" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="M6" s="3">
         <v>45399</v>
@@ -1287,10 +1286,10 @@
         <v>16000000</v>
       </c>
       <c r="O6" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="P6" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.2">
@@ -1298,37 +1297,37 @@
         <v>15</v>
       </c>
       <c r="B7" t="s">
+        <v>181</v>
+      </c>
+      <c r="C7" t="s">
+        <v>37</v>
+      </c>
+      <c r="D7" t="s">
         <v>38</v>
-      </c>
-      <c r="C7" t="s">
-        <v>39</v>
-      </c>
-      <c r="D7" t="s">
-        <v>40</v>
       </c>
       <c r="E7">
         <v>2</v>
       </c>
       <c r="F7" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="G7" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="H7" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I7" t="s">
+        <v>118</v>
+      </c>
+      <c r="J7" t="s">
+        <v>121</v>
+      </c>
+      <c r="K7" t="s">
         <v>123</v>
       </c>
-      <c r="J7" t="s">
-        <v>126</v>
-      </c>
-      <c r="K7" t="s">
-        <v>128</v>
-      </c>
       <c r="L7" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="M7" s="3">
         <v>45415</v>
@@ -1337,7 +1336,7 @@
         <v>24000000</v>
       </c>
       <c r="O7" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.2">
@@ -1345,37 +1344,37 @@
         <v>16</v>
       </c>
       <c r="B8" t="s">
-        <v>59</v>
+        <v>179</v>
       </c>
       <c r="C8" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D8" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E8">
         <v>2</v>
       </c>
       <c r="F8" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="G8" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="H8" t="s">
+        <v>125</v>
+      </c>
+      <c r="I8" t="s">
+        <v>128</v>
+      </c>
+      <c r="J8" t="s">
         <v>130</v>
       </c>
-      <c r="I8" t="s">
+      <c r="K8" t="s">
         <v>133</v>
       </c>
-      <c r="J8" t="s">
+      <c r="L8" t="s">
         <v>135</v>
-      </c>
-      <c r="K8" t="s">
-        <v>138</v>
-      </c>
-      <c r="L8" t="s">
-        <v>140</v>
       </c>
       <c r="M8" s="3">
         <v>45427</v>
@@ -1384,7 +1383,7 @@
         <v>16000000</v>
       </c>
       <c r="O8" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.2">
@@ -1392,37 +1391,37 @@
         <v>17</v>
       </c>
       <c r="B9" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C9" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D9" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E9">
         <v>3</v>
       </c>
       <c r="F9" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="G9" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="H9" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="I9" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="J9" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="K9" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="L9" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="M9" s="3">
         <v>45443</v>
@@ -1431,10 +1430,10 @@
         <v>180000</v>
       </c>
       <c r="O9" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="P9" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.2">
@@ -1442,37 +1441,37 @@
         <v>18</v>
       </c>
       <c r="B10" t="s">
-        <v>47</v>
+        <v>180</v>
       </c>
       <c r="C10" t="s">
         <v>34</v>
       </c>
       <c r="D10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E10">
         <v>5</v>
       </c>
       <c r="F10" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="G10" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="H10" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="I10" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="J10" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="K10" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="L10" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="M10" s="3">
         <v>45432</v>
@@ -1481,10 +1480,10 @@
         <v>35000000</v>
       </c>
       <c r="O10" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="P10" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.2">
@@ -1492,37 +1491,37 @@
         <v>19</v>
       </c>
       <c r="B11" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C11" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="D11" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E11" s="5">
         <v>2</v>
       </c>
       <c r="F11" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="G11" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="H11" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="I11" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="J11" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="K11" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="L11" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="M11" s="3">
         <v>45444</v>
@@ -1531,7 +1530,7 @@
         <v>2900000</v>
       </c>
       <c r="O11" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.2">
@@ -1539,37 +1538,37 @@
         <v>20</v>
       </c>
       <c r="B12" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C12" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="D12" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E12" s="5">
         <v>2</v>
       </c>
       <c r="F12" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="G12" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="H12" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="I12" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="J12" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="K12" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="L12" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="M12" s="3">
         <v>45453</v>
@@ -1578,7 +1577,7 @@
         <v>2900000</v>
       </c>
       <c r="O12" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.2">
@@ -1586,37 +1585,37 @@
         <v>21</v>
       </c>
       <c r="B13" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C13" t="s">
         <v>34</v>
       </c>
       <c r="D13" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E13">
         <v>5</v>
       </c>
       <c r="F13" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="G13" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="H13" t="s">
+        <v>117</v>
+      </c>
+      <c r="I13" t="s">
+        <v>118</v>
+      </c>
+      <c r="J13" t="s">
+        <v>121</v>
+      </c>
+      <c r="K13" t="s">
         <v>122</v>
       </c>
-      <c r="I13" t="s">
-        <v>123</v>
-      </c>
-      <c r="J13" t="s">
-        <v>126</v>
-      </c>
-      <c r="K13" t="s">
-        <v>127</v>
-      </c>
       <c r="L13" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="M13" s="3">
         <v>45455</v>
@@ -1625,10 +1624,10 @@
         <v>21000000</v>
       </c>
       <c r="O13" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="P13" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.2">
@@ -1636,37 +1635,37 @@
         <v>22</v>
       </c>
       <c r="B14" t="s">
-        <v>82</v>
+        <v>182</v>
       </c>
       <c r="C14" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="D14" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E14">
         <v>3</v>
       </c>
       <c r="F14" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="G14" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="H14" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I14" t="s">
+        <v>118</v>
+      </c>
+      <c r="J14" t="s">
+        <v>131</v>
+      </c>
+      <c r="K14" t="s">
         <v>123</v>
       </c>
-      <c r="J14" t="s">
-        <v>136</v>
-      </c>
-      <c r="K14" t="s">
-        <v>128</v>
-      </c>
       <c r="L14" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="M14" s="3">
         <v>45474</v>
@@ -1675,10 +1674,10 @@
         <v>14000000</v>
       </c>
       <c r="O14" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="P14" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.2">
@@ -1686,37 +1685,37 @@
         <v>23</v>
       </c>
       <c r="B15" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="C15" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="D15" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E15">
         <v>5</v>
       </c>
       <c r="F15" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="G15" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="H15" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="I15" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="J15" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="K15" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="L15" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="M15" s="3">
         <v>45483</v>
@@ -1725,10 +1724,10 @@
         <v>6100000</v>
       </c>
       <c r="O15" s="5" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="P15" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.2">
@@ -1736,37 +1735,37 @@
         <v>24</v>
       </c>
       <c r="B16" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="C16" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="D16" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="E16">
         <v>2</v>
       </c>
       <c r="F16" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="G16" t="s">
+        <v>137</v>
+      </c>
+      <c r="H16" t="s">
+        <v>139</v>
+      </c>
+      <c r="I16" t="s">
+        <v>118</v>
+      </c>
+      <c r="J16" t="s">
+        <v>131</v>
+      </c>
+      <c r="K16" t="s">
+        <v>122</v>
+      </c>
+      <c r="L16" t="s">
         <v>142</v>
-      </c>
-      <c r="H16" t="s">
-        <v>144</v>
-      </c>
-      <c r="I16" t="s">
-        <v>123</v>
-      </c>
-      <c r="J16" t="s">
-        <v>136</v>
-      </c>
-      <c r="K16" t="s">
-        <v>127</v>
-      </c>
-      <c r="L16" t="s">
-        <v>147</v>
       </c>
       <c r="M16" s="3">
         <v>45514</v>
@@ -1775,7 +1774,7 @@
         <v>11000000</v>
       </c>
       <c r="O16" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.2">
@@ -1783,37 +1782,37 @@
         <v>25</v>
       </c>
       <c r="B17" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C17" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D17" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E17">
         <v>5</v>
       </c>
       <c r="F17" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="G17" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="H17" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="I17" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="J17" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="K17" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="L17" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="M17" s="3">
         <v>45563</v>
@@ -1822,10 +1821,10 @@
         <v>180000</v>
       </c>
       <c r="O17" s="5" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="P17" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.2">
@@ -1833,37 +1832,37 @@
         <v>26</v>
       </c>
       <c r="B18" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="C18" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="D18" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="E18">
         <v>5</v>
       </c>
       <c r="F18" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="G18" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="H18" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="I18" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="J18" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="K18" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="L18" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="M18" s="3">
         <v>45584</v>
@@ -1872,10 +1871,10 @@
         <v>2250000</v>
       </c>
       <c r="O18" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="P18" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.2">
@@ -1883,37 +1882,37 @@
         <v>27</v>
       </c>
       <c r="B19" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="C19" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="D19" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="E19">
         <v>5</v>
       </c>
       <c r="F19" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="G19" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="H19" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="I19" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="J19" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="K19" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="L19" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="M19" s="3">
         <v>45593</v>
@@ -1922,10 +1921,10 @@
         <v>2250000</v>
       </c>
       <c r="O19" s="5" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="P19" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.2">
@@ -1933,37 +1932,37 @@
         <v>28</v>
       </c>
       <c r="B20" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="C20" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="D20" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E20">
         <v>2</v>
       </c>
       <c r="F20" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="G20" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="H20" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="I20" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="J20" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="K20" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="L20" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="M20" s="3">
         <v>45606</v>
@@ -1972,7 +1971,7 @@
         <v>6100000</v>
       </c>
       <c r="O20" s="5" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.2">
@@ -1980,37 +1979,37 @@
         <v>29</v>
       </c>
       <c r="B21" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C21" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D21" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="E21">
         <v>5</v>
       </c>
       <c r="F21" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="G21" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="H21" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="I21" t="s">
+        <v>127</v>
+      </c>
+      <c r="J21" t="s">
+        <v>131</v>
+      </c>
+      <c r="K21" t="s">
         <v>132</v>
       </c>
-      <c r="J21" t="s">
-        <v>136</v>
-      </c>
-      <c r="K21" t="s">
-        <v>137</v>
-      </c>
       <c r="L21" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="M21" s="3">
         <v>45615</v>
@@ -2019,10 +2018,10 @@
         <v>25000000</v>
       </c>
       <c r="O21" s="5" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="P21" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.2">
@@ -2030,37 +2029,37 @@
         <v>30</v>
       </c>
       <c r="B22" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C22" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="D22" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E22">
         <v>2</v>
       </c>
       <c r="F22" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="G22" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="H22" t="s">
+        <v>156</v>
+      </c>
+      <c r="I22" t="s">
         <v>161</v>
       </c>
-      <c r="I22" t="s">
+      <c r="J22" t="s">
+        <v>165</v>
+      </c>
+      <c r="K22" t="s">
         <v>166</v>
       </c>
-      <c r="J22" t="s">
+      <c r="L22" t="s">
         <v>170</v>
-      </c>
-      <c r="K22" t="s">
-        <v>171</v>
-      </c>
-      <c r="L22" t="s">
-        <v>175</v>
       </c>
       <c r="M22" s="3">
         <v>45623</v>
@@ -2069,7 +2068,7 @@
         <v>120000</v>
       </c>
       <c r="O22" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.2">
@@ -2077,37 +2076,37 @@
         <v>31</v>
       </c>
       <c r="B23" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="C23" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D23" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E23">
         <v>4</v>
       </c>
       <c r="F23" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="G23" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="H23" t="s">
+        <v>156</v>
+      </c>
+      <c r="I23" t="s">
+        <v>162</v>
+      </c>
+      <c r="J23" t="s">
         <v>161</v>
       </c>
-      <c r="I23" t="s">
-        <v>167</v>
-      </c>
-      <c r="J23" t="s">
+      <c r="K23" t="s">
         <v>166</v>
       </c>
-      <c r="K23" t="s">
-        <v>171</v>
-      </c>
       <c r="L23" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="M23" s="3">
         <v>45628</v>
@@ -2116,7 +2115,7 @@
         <v>1800000</v>
       </c>
       <c r="O23" s="5" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.2">
@@ -2124,37 +2123,37 @@
         <v>32</v>
       </c>
       <c r="B24" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="C24" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="D24" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E24">
         <v>4</v>
       </c>
       <c r="F24" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="G24" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="H24" t="s">
+        <v>156</v>
+      </c>
+      <c r="I24" t="s">
         <v>161</v>
       </c>
-      <c r="I24" t="s">
-        <v>166</v>
-      </c>
       <c r="J24" t="s">
+        <v>165</v>
+      </c>
+      <c r="K24" t="s">
+        <v>169</v>
+      </c>
+      <c r="L24" t="s">
         <v>170</v>
-      </c>
-      <c r="K24" t="s">
-        <v>174</v>
-      </c>
-      <c r="L24" t="s">
-        <v>175</v>
       </c>
       <c r="M24" s="3">
         <v>45636</v>
@@ -2163,7 +2162,7 @@
         <v>150000</v>
       </c>
       <c r="O24" s="5" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.2">
@@ -2171,37 +2170,37 @@
         <v>33</v>
       </c>
       <c r="B25" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C25" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D25" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E25">
         <v>3</v>
       </c>
       <c r="F25" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="G25" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="H25" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="I25" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="J25" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="K25" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="L25" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="M25" s="3">
         <v>45638</v>
@@ -2210,10 +2209,10 @@
         <v>180000</v>
       </c>
       <c r="O25" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="P25" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Script v1 and removed name column from data
</commit_message>
<xml_diff>
--- a/data/Dummy data.xlsx
+++ b/data/Dummy data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xav/Documents/GitHub/privy-snipeit/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DB5F775-EFB5-A346-940D-F023E0A92EDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04E12CF0-4FF0-D54F-A737-0F75BF6290BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="28800" windowHeight="16340" xr2:uid="{E460BB3F-4FF0-1D4F-8F63-FB9F8008A7DA}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="168">
   <si>
     <t>Asset Tag</t>
   </si>
@@ -67,9 +67,6 @@
     <t>Location</t>
   </si>
   <si>
-    <t>Assigned To</t>
-  </si>
-  <si>
     <t>A0002</t>
   </si>
   <si>
@@ -148,9 +145,6 @@
     <t>Dell</t>
   </si>
   <si>
-    <t>Sarah</t>
-  </si>
-  <si>
     <t xml:space="preserve">Laptop </t>
   </si>
   <si>
@@ -172,15 +166,9 @@
     <t>LNO1223</t>
   </si>
   <si>
-    <t>Yaya</t>
-  </si>
-  <si>
     <t>APP1213</t>
   </si>
   <si>
-    <t>Yuan</t>
-  </si>
-  <si>
     <t>EliteBook 840 G11</t>
   </si>
   <si>
@@ -190,9 +178,6 @@
     <t>HHP2232</t>
   </si>
   <si>
-    <t>Jojo</t>
-  </si>
-  <si>
     <t>Galaxy S24</t>
   </si>
   <si>
@@ -293,36 +278,6 @@
   </si>
   <si>
     <t>MCF390</t>
-  </si>
-  <si>
-    <t>Rina</t>
-  </si>
-  <si>
-    <t>Budi</t>
-  </si>
-  <si>
-    <t>Juan</t>
-  </si>
-  <si>
-    <t>Afi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ayu </t>
-  </si>
-  <si>
-    <t>Kina</t>
-  </si>
-  <si>
-    <t>Fajar</t>
-  </si>
-  <si>
-    <t>Salman</t>
-  </si>
-  <si>
-    <t>Rian</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dimas </t>
   </si>
   <si>
     <t>Mac Address</t>
@@ -1013,22 +968,22 @@
         <v>5</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>97</v>
+        <v>82</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>98</v>
+        <v>83</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>99</v>
+        <v>84</v>
       </c>
       <c r="L1" s="6" t="s">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="M1" s="6" t="s">
         <v>6</v>
@@ -1039,48 +994,46 @@
       <c r="O1" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="P1" s="6" t="s">
-        <v>9</v>
-      </c>
+      <c r="P1" s="6"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="2"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>178</v>
+        <v>163</v>
       </c>
       <c r="C2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D2" t="s">
         <v>34</v>
-      </c>
-      <c r="D2" t="s">
-        <v>35</v>
       </c>
       <c r="E2">
         <v>5</v>
       </c>
       <c r="F2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="G2" t="s">
+        <v>88</v>
+      </c>
+      <c r="H2" t="s">
+        <v>98</v>
+      </c>
+      <c r="I2" t="s">
         <v>103</v>
       </c>
-      <c r="H2" t="s">
-        <v>113</v>
-      </c>
-      <c r="I2" t="s">
-        <v>118</v>
-      </c>
       <c r="J2" t="s">
-        <v>121</v>
+        <v>106</v>
       </c>
       <c r="K2" t="s">
-        <v>122</v>
+        <v>107</v>
       </c>
       <c r="L2" t="s">
-        <v>174</v>
+        <v>159</v>
       </c>
       <c r="M2" s="3">
         <v>45294</v>
@@ -1089,48 +1042,45 @@
         <v>13000000</v>
       </c>
       <c r="O2" t="s">
-        <v>101</v>
-      </c>
-      <c r="P2" t="s">
-        <v>36</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C3" t="s">
         <v>51</v>
       </c>
-      <c r="C3" t="s">
-        <v>56</v>
-      </c>
       <c r="D3" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="E3">
         <v>2</v>
       </c>
       <c r="F3" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="G3" t="s">
-        <v>108</v>
+        <v>93</v>
       </c>
       <c r="H3" t="s">
-        <v>124</v>
+        <v>109</v>
       </c>
       <c r="I3" t="s">
-        <v>126</v>
+        <v>111</v>
       </c>
       <c r="J3" t="s">
-        <v>129</v>
+        <v>114</v>
       </c>
       <c r="K3" t="s">
-        <v>132</v>
+        <v>117</v>
       </c>
       <c r="L3" t="s">
-        <v>134</v>
+        <v>119</v>
       </c>
       <c r="M3" s="3">
         <v>45316</v>
@@ -1139,45 +1089,45 @@
         <v>12000000</v>
       </c>
       <c r="O3" t="s">
-        <v>102</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D4" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E4">
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="G4" t="s">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="H4" t="s">
-        <v>114</v>
+        <v>99</v>
       </c>
       <c r="I4" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="J4" t="s">
-        <v>121</v>
+        <v>106</v>
       </c>
       <c r="K4" t="s">
-        <v>122</v>
+        <v>107</v>
       </c>
       <c r="L4" t="s">
-        <v>175</v>
+        <v>160</v>
       </c>
       <c r="M4" s="3">
         <v>45325</v>
@@ -1186,48 +1136,45 @@
         <v>19000000</v>
       </c>
       <c r="O4" t="s">
-        <v>102</v>
-      </c>
-      <c r="P4" t="s">
-        <v>44</v>
+        <v>87</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="C5" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="D5" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="E5">
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="G5" t="s">
+        <v>97</v>
+      </c>
+      <c r="H5" t="s">
+        <v>109</v>
+      </c>
+      <c r="I5" t="s">
         <v>112</v>
       </c>
-      <c r="H5" t="s">
-        <v>124</v>
-      </c>
-      <c r="I5" t="s">
-        <v>127</v>
-      </c>
       <c r="J5" t="s">
-        <v>121</v>
+        <v>106</v>
       </c>
       <c r="K5" t="s">
-        <v>132</v>
+        <v>117</v>
       </c>
       <c r="L5" t="s">
-        <v>134</v>
+        <v>119</v>
       </c>
       <c r="M5" s="3">
         <v>45373</v>
@@ -1236,48 +1183,45 @@
         <v>20000000</v>
       </c>
       <c r="O5" t="s">
-        <v>102</v>
-      </c>
-      <c r="P5" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>179</v>
+        <v>164</v>
       </c>
       <c r="C6" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="D6" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E6">
         <v>5</v>
       </c>
       <c r="F6" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="G6" t="s">
+        <v>95</v>
+      </c>
+      <c r="H6" t="s">
         <v>110</v>
       </c>
-      <c r="H6" t="s">
-        <v>125</v>
-      </c>
       <c r="I6" t="s">
-        <v>128</v>
+        <v>113</v>
       </c>
       <c r="J6" t="s">
-        <v>129</v>
+        <v>114</v>
       </c>
       <c r="K6" t="s">
-        <v>133</v>
+        <v>118</v>
       </c>
       <c r="L6" t="s">
-        <v>135</v>
+        <v>120</v>
       </c>
       <c r="M6" s="3">
         <v>45399</v>
@@ -1286,48 +1230,45 @@
         <v>16000000</v>
       </c>
       <c r="O6" t="s">
-        <v>101</v>
-      </c>
-      <c r="P6" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>181</v>
+        <v>166</v>
       </c>
       <c r="C7" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D7" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E7">
         <v>2</v>
       </c>
       <c r="F7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G7" t="s">
-        <v>105</v>
+        <v>90</v>
       </c>
       <c r="H7" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
       <c r="I7" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="J7" t="s">
-        <v>121</v>
+        <v>106</v>
       </c>
       <c r="K7" t="s">
-        <v>123</v>
+        <v>108</v>
       </c>
       <c r="L7" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="M7" s="3">
         <v>45415</v>
@@ -1336,45 +1277,45 @@
         <v>24000000</v>
       </c>
       <c r="O7" t="s">
-        <v>102</v>
+        <v>87</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>179</v>
+        <v>164</v>
       </c>
       <c r="C8" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="D8" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E8">
         <v>2</v>
       </c>
       <c r="F8" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="G8" t="s">
-        <v>111</v>
+        <v>96</v>
       </c>
       <c r="H8" t="s">
-        <v>125</v>
+        <v>110</v>
       </c>
       <c r="I8" t="s">
-        <v>128</v>
+        <v>113</v>
       </c>
       <c r="J8" t="s">
-        <v>130</v>
+        <v>115</v>
       </c>
       <c r="K8" t="s">
-        <v>133</v>
+        <v>118</v>
       </c>
       <c r="L8" t="s">
-        <v>135</v>
+        <v>120</v>
       </c>
       <c r="M8" s="3">
         <v>45427</v>
@@ -1383,45 +1324,45 @@
         <v>16000000</v>
       </c>
       <c r="O8" t="s">
-        <v>102</v>
+        <v>87</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C9" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="D9" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="E9">
         <v>3</v>
       </c>
       <c r="F9" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="G9" t="s">
-        <v>146</v>
+        <v>131</v>
       </c>
       <c r="H9" t="s">
-        <v>156</v>
+        <v>141</v>
       </c>
       <c r="I9" t="s">
-        <v>159</v>
+        <v>144</v>
       </c>
       <c r="J9" t="s">
-        <v>163</v>
+        <v>148</v>
       </c>
       <c r="K9" t="s">
-        <v>166</v>
+        <v>151</v>
       </c>
       <c r="L9" t="s">
-        <v>170</v>
+        <v>155</v>
       </c>
       <c r="M9" s="3">
         <v>45443</v>
@@ -1430,48 +1371,45 @@
         <v>180000</v>
       </c>
       <c r="O9" t="s">
-        <v>101</v>
-      </c>
-      <c r="P9" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B10" t="s">
-        <v>180</v>
+        <v>165</v>
       </c>
       <c r="C10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D10" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E10">
         <v>5</v>
       </c>
       <c r="F10" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="G10" t="s">
-        <v>106</v>
+        <v>91</v>
       </c>
       <c r="H10" t="s">
-        <v>116</v>
+        <v>101</v>
       </c>
       <c r="I10" t="s">
-        <v>119</v>
+        <v>104</v>
       </c>
       <c r="J10" t="s">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="K10" t="s">
-        <v>123</v>
+        <v>108</v>
       </c>
       <c r="L10" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="M10" s="3">
         <v>45432</v>
@@ -1480,48 +1418,45 @@
         <v>35000000</v>
       </c>
       <c r="O10" t="s">
-        <v>101</v>
-      </c>
-      <c r="P10" t="s">
-        <v>46</v>
+        <v>86</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B11" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="C11" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="D11" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E11" s="5">
         <v>2</v>
       </c>
       <c r="F11" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="G11" t="s">
-        <v>147</v>
+        <v>132</v>
       </c>
       <c r="H11" t="s">
-        <v>157</v>
+        <v>142</v>
       </c>
       <c r="I11" t="s">
-        <v>160</v>
+        <v>145</v>
       </c>
       <c r="J11" t="s">
-        <v>159</v>
+        <v>144</v>
       </c>
       <c r="K11" t="s">
-        <v>167</v>
+        <v>152</v>
       </c>
       <c r="L11" t="s">
-        <v>170</v>
+        <v>155</v>
       </c>
       <c r="M11" s="3">
         <v>45444</v>
@@ -1530,45 +1465,45 @@
         <v>2900000</v>
       </c>
       <c r="O11" t="s">
-        <v>102</v>
+        <v>87</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B12" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="C12" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="D12" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E12" s="5">
         <v>2</v>
       </c>
       <c r="F12" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="G12" t="s">
-        <v>148</v>
+        <v>133</v>
       </c>
       <c r="H12" t="s">
-        <v>157</v>
+        <v>142</v>
       </c>
       <c r="I12" t="s">
-        <v>160</v>
+        <v>145</v>
       </c>
       <c r="J12" t="s">
-        <v>159</v>
+        <v>144</v>
       </c>
       <c r="K12" t="s">
-        <v>167</v>
+        <v>152</v>
       </c>
       <c r="L12" t="s">
-        <v>170</v>
+        <v>155</v>
       </c>
       <c r="M12" s="3">
         <v>45453</v>
@@ -1577,45 +1512,45 @@
         <v>2900000</v>
       </c>
       <c r="O12" t="s">
-        <v>102</v>
+        <v>87</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B13" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C13" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D13" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E13">
         <v>5</v>
       </c>
       <c r="F13" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="G13" t="s">
+        <v>92</v>
+      </c>
+      <c r="H13" t="s">
+        <v>102</v>
+      </c>
+      <c r="I13" t="s">
+        <v>103</v>
+      </c>
+      <c r="J13" t="s">
+        <v>106</v>
+      </c>
+      <c r="K13" t="s">
         <v>107</v>
       </c>
-      <c r="H13" t="s">
-        <v>117</v>
-      </c>
-      <c r="I13" t="s">
-        <v>118</v>
-      </c>
-      <c r="J13" t="s">
-        <v>121</v>
-      </c>
-      <c r="K13" t="s">
-        <v>122</v>
-      </c>
       <c r="L13" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="M13" s="3">
         <v>45455</v>
@@ -1624,48 +1559,45 @@
         <v>21000000</v>
       </c>
       <c r="O13" t="s">
-        <v>101</v>
-      </c>
-      <c r="P13" t="s">
-        <v>50</v>
+        <v>86</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B14" t="s">
-        <v>182</v>
+        <v>167</v>
       </c>
       <c r="C14" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="D14" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E14">
         <v>3</v>
       </c>
       <c r="F14" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="G14" t="s">
-        <v>136</v>
+        <v>121</v>
       </c>
       <c r="H14" t="s">
-        <v>138</v>
+        <v>123</v>
       </c>
       <c r="I14" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="J14" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="K14" t="s">
-        <v>123</v>
+        <v>108</v>
       </c>
       <c r="L14" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="M14" s="3">
         <v>45474</v>
@@ -1674,48 +1606,45 @@
         <v>14000000</v>
       </c>
       <c r="O14" t="s">
-        <v>102</v>
-      </c>
-      <c r="P14" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B15" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="C15" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="D15" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E15">
         <v>5</v>
       </c>
       <c r="F15" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="G15" t="s">
-        <v>149</v>
+        <v>134</v>
       </c>
       <c r="H15" t="s">
-        <v>157</v>
+        <v>142</v>
       </c>
       <c r="I15" t="s">
-        <v>160</v>
+        <v>145</v>
       </c>
       <c r="J15" t="s">
-        <v>159</v>
+        <v>144</v>
       </c>
       <c r="K15" t="s">
-        <v>167</v>
+        <v>152</v>
       </c>
       <c r="L15" t="s">
-        <v>170</v>
+        <v>155</v>
       </c>
       <c r="M15" s="3">
         <v>45483</v>
@@ -1724,48 +1653,45 @@
         <v>6100000</v>
       </c>
       <c r="O15" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="P15" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B16" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C16" t="s">
-        <v>177</v>
+        <v>162</v>
       </c>
       <c r="D16" t="s">
-        <v>140</v>
+        <v>125</v>
       </c>
       <c r="E16">
         <v>2</v>
       </c>
       <c r="F16" t="s">
-        <v>141</v>
+        <v>126</v>
       </c>
       <c r="G16" t="s">
-        <v>137</v>
+        <v>122</v>
       </c>
       <c r="H16" t="s">
-        <v>139</v>
+        <v>124</v>
       </c>
       <c r="I16" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="J16" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="K16" t="s">
-        <v>122</v>
+        <v>107</v>
       </c>
       <c r="L16" t="s">
-        <v>142</v>
+        <v>127</v>
       </c>
       <c r="M16" s="3">
         <v>45514</v>
@@ -1774,45 +1700,45 @@
         <v>11000000</v>
       </c>
       <c r="O16" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B17" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C17" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="D17" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="E17">
         <v>5</v>
       </c>
       <c r="F17" t="s">
-        <v>143</v>
+        <v>128</v>
       </c>
       <c r="G17" t="s">
-        <v>150</v>
+        <v>135</v>
       </c>
       <c r="H17" t="s">
-        <v>156</v>
+        <v>141</v>
       </c>
       <c r="I17" t="s">
-        <v>159</v>
+        <v>144</v>
       </c>
       <c r="J17" t="s">
-        <v>163</v>
+        <v>148</v>
       </c>
       <c r="K17" t="s">
-        <v>166</v>
+        <v>151</v>
       </c>
       <c r="L17" t="s">
-        <v>170</v>
+        <v>155</v>
       </c>
       <c r="M17" s="3">
         <v>45563</v>
@@ -1821,48 +1747,45 @@
         <v>180000</v>
       </c>
       <c r="O17" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="P17" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B18" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="C18" t="s">
-        <v>144</v>
+        <v>129</v>
       </c>
       <c r="D18" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="E18">
         <v>5</v>
       </c>
       <c r="F18" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="G18" t="s">
-        <v>172</v>
+        <v>157</v>
       </c>
       <c r="H18" t="s">
-        <v>158</v>
+        <v>143</v>
       </c>
       <c r="I18" t="s">
-        <v>126</v>
+        <v>111</v>
       </c>
       <c r="J18" t="s">
-        <v>164</v>
+        <v>149</v>
       </c>
       <c r="K18" t="s">
-        <v>168</v>
+        <v>153</v>
       </c>
       <c r="L18" t="s">
-        <v>171</v>
+        <v>156</v>
       </c>
       <c r="M18" s="3">
         <v>45584</v>
@@ -1871,48 +1794,45 @@
         <v>2250000</v>
       </c>
       <c r="O18" t="s">
-        <v>102</v>
-      </c>
-      <c r="P18" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B19" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="C19" t="s">
-        <v>144</v>
+        <v>129</v>
       </c>
       <c r="D19" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="E19">
         <v>5</v>
       </c>
       <c r="F19" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="G19" t="s">
-        <v>173</v>
+        <v>158</v>
       </c>
       <c r="H19" t="s">
-        <v>158</v>
+        <v>143</v>
       </c>
       <c r="I19" t="s">
-        <v>126</v>
+        <v>111</v>
       </c>
       <c r="J19" t="s">
-        <v>164</v>
+        <v>149</v>
       </c>
       <c r="K19" t="s">
-        <v>168</v>
+        <v>153</v>
       </c>
       <c r="L19" t="s">
-        <v>171</v>
+        <v>156</v>
       </c>
       <c r="M19" s="3">
         <v>45593</v>
@@ -1921,48 +1841,45 @@
         <v>2250000</v>
       </c>
       <c r="O19" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="P19" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B20" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="C20" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="D20" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E20">
         <v>2</v>
       </c>
       <c r="F20" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="G20" t="s">
-        <v>151</v>
+        <v>136</v>
       </c>
       <c r="H20" t="s">
-        <v>157</v>
+        <v>142</v>
       </c>
       <c r="I20" t="s">
-        <v>160</v>
+        <v>145</v>
       </c>
       <c r="J20" t="s">
-        <v>159</v>
+        <v>144</v>
       </c>
       <c r="K20" t="s">
-        <v>167</v>
+        <v>152</v>
       </c>
       <c r="L20" t="s">
-        <v>170</v>
+        <v>155</v>
       </c>
       <c r="M20" s="3">
         <v>45606</v>
@@ -1971,45 +1888,45 @@
         <v>6100000</v>
       </c>
       <c r="O20" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B21" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="C21" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="D21" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="E21">
         <v>5</v>
       </c>
       <c r="F21" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="G21" t="s">
+        <v>94</v>
+      </c>
+      <c r="H21" t="s">
         <v>109</v>
       </c>
-      <c r="H21" t="s">
-        <v>124</v>
-      </c>
       <c r="I21" t="s">
-        <v>127</v>
+        <v>112</v>
       </c>
       <c r="J21" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="K21" t="s">
-        <v>132</v>
+        <v>117</v>
       </c>
       <c r="L21" t="s">
-        <v>134</v>
+        <v>119</v>
       </c>
       <c r="M21" s="3">
         <v>45615</v>
@@ -2018,48 +1935,45 @@
         <v>25000000</v>
       </c>
       <c r="O21" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="P21" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B22" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C22" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="D22" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E22">
         <v>2</v>
       </c>
       <c r="F22" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="G22" t="s">
-        <v>152</v>
+        <v>137</v>
       </c>
       <c r="H22" t="s">
-        <v>156</v>
+        <v>141</v>
       </c>
       <c r="I22" t="s">
-        <v>161</v>
+        <v>146</v>
       </c>
       <c r="J22" t="s">
-        <v>165</v>
+        <v>150</v>
       </c>
       <c r="K22" t="s">
-        <v>166</v>
+        <v>151</v>
       </c>
       <c r="L22" t="s">
-        <v>170</v>
+        <v>155</v>
       </c>
       <c r="M22" s="3">
         <v>45623</v>
@@ -2068,45 +1982,45 @@
         <v>120000</v>
       </c>
       <c r="O22" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B23" t="s">
-        <v>145</v>
+        <v>130</v>
       </c>
       <c r="C23" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="D23" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="E23">
         <v>4</v>
       </c>
       <c r="F23" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="G23" t="s">
-        <v>153</v>
+        <v>138</v>
       </c>
       <c r="H23" t="s">
-        <v>156</v>
+        <v>141</v>
       </c>
       <c r="I23" t="s">
-        <v>162</v>
+        <v>147</v>
       </c>
       <c r="J23" t="s">
-        <v>161</v>
+        <v>146</v>
       </c>
       <c r="K23" t="s">
-        <v>166</v>
+        <v>151</v>
       </c>
       <c r="L23" t="s">
-        <v>170</v>
+        <v>155</v>
       </c>
       <c r="M23" s="3">
         <v>45628</v>
@@ -2115,45 +2029,45 @@
         <v>1800000</v>
       </c>
       <c r="O23" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B24" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="C24" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="D24" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="E24">
         <v>4</v>
       </c>
       <c r="F24" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="G24" t="s">
+        <v>139</v>
+      </c>
+      <c r="H24" t="s">
+        <v>141</v>
+      </c>
+      <c r="I24" t="s">
+        <v>146</v>
+      </c>
+      <c r="J24" t="s">
+        <v>150</v>
+      </c>
+      <c r="K24" t="s">
         <v>154</v>
       </c>
-      <c r="H24" t="s">
-        <v>156</v>
-      </c>
-      <c r="I24" t="s">
-        <v>161</v>
-      </c>
-      <c r="J24" t="s">
-        <v>165</v>
-      </c>
-      <c r="K24" t="s">
-        <v>169</v>
-      </c>
       <c r="L24" t="s">
-        <v>170</v>
+        <v>155</v>
       </c>
       <c r="M24" s="3">
         <v>45636</v>
@@ -2162,45 +2076,45 @@
         <v>150000</v>
       </c>
       <c r="O24" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.2">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B25" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C25" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="D25" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="E25">
         <v>3</v>
       </c>
       <c r="F25" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="G25" t="s">
+        <v>140</v>
+      </c>
+      <c r="H25" t="s">
+        <v>141</v>
+      </c>
+      <c r="I25" t="s">
+        <v>144</v>
+      </c>
+      <c r="J25" t="s">
+        <v>148</v>
+      </c>
+      <c r="K25" t="s">
+        <v>151</v>
+      </c>
+      <c r="L25" t="s">
         <v>155</v>
-      </c>
-      <c r="H25" t="s">
-        <v>156</v>
-      </c>
-      <c r="I25" t="s">
-        <v>159</v>
-      </c>
-      <c r="J25" t="s">
-        <v>163</v>
-      </c>
-      <c r="K25" t="s">
-        <v>166</v>
-      </c>
-      <c r="L25" t="s">
-        <v>170</v>
       </c>
       <c r="M25" s="3">
         <v>45638</v>
@@ -2209,10 +2123,7 @@
         <v>180000</v>
       </c>
       <c r="O25" t="s">
-        <v>102</v>
-      </c>
-      <c r="P25" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Change data type for purchase date and delete column for assign to
</commit_message>
<xml_diff>
--- a/data/Dummy data.xlsx
+++ b/data/Dummy data.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11028"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xav/Documents/GitHub/privy-snipeit/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nadhifaazka/Documents/GitHub/privy-snipeit/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DB5F775-EFB5-A346-940D-F023E0A92EDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAD0399D-39EC-5344-AE64-3D81AC7947B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="28800" windowHeight="16340" xr2:uid="{E460BB3F-4FF0-1D4F-8F63-FB9F8008A7DA}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16340" xr2:uid="{E460BB3F-4FF0-1D4F-8F63-FB9F8008A7DA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$P$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$O$25</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="168">
   <si>
     <t>Asset Tag</t>
   </si>
@@ -67,9 +67,6 @@
     <t>Location</t>
   </si>
   <si>
-    <t>Assigned To</t>
-  </si>
-  <si>
     <t>A0002</t>
   </si>
   <si>
@@ -148,9 +145,6 @@
     <t>Dell</t>
   </si>
   <si>
-    <t>Sarah</t>
-  </si>
-  <si>
     <t xml:space="preserve">Laptop </t>
   </si>
   <si>
@@ -172,15 +166,9 @@
     <t>LNO1223</t>
   </si>
   <si>
-    <t>Yaya</t>
-  </si>
-  <si>
     <t>APP1213</t>
   </si>
   <si>
-    <t>Yuan</t>
-  </si>
-  <si>
     <t>EliteBook 840 G11</t>
   </si>
   <si>
@@ -190,9 +178,6 @@
     <t>HHP2232</t>
   </si>
   <si>
-    <t>Jojo</t>
-  </si>
-  <si>
     <t>Galaxy S24</t>
   </si>
   <si>
@@ -293,36 +278,6 @@
   </si>
   <si>
     <t>MCF390</t>
-  </si>
-  <si>
-    <t>Rina</t>
-  </si>
-  <si>
-    <t>Budi</t>
-  </si>
-  <si>
-    <t>Juan</t>
-  </si>
-  <si>
-    <t>Afi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ayu </t>
-  </si>
-  <si>
-    <t>Kina</t>
-  </si>
-  <si>
-    <t>Fajar</t>
-  </si>
-  <si>
-    <t>Salman</t>
-  </si>
-  <si>
-    <t>Rian</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dimas </t>
   </si>
   <si>
     <t>Mac Address</t>
@@ -593,6 +548,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
+  </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -654,10 +612,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -676,9 +634,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -716,7 +674,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -822,7 +780,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -964,7 +922,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -972,7 +930,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61CE36BB-B836-FE48-96B8-B2CA2E34C478}">
-  <dimension ref="A1:R25"/>
+  <dimension ref="A1:Q25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -990,1233 +948,1187 @@
     <col min="13" max="13" width="14" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="14.1640625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="H1" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="I1" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="J1" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="K1" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="L1" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="M1" s="6" t="s">
+      <c r="G1" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="L1" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="M1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="N1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="O1" s="6" t="s">
+      <c r="O1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="P1" s="6" t="s">
+      <c r="P1" s="1"/>
+      <c r="Q1" s="2"/>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>9</v>
       </c>
-      <c r="Q1" s="1"/>
-      <c r="R1" s="2"/>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>10</v>
-      </c>
       <c r="B2" t="s">
-        <v>178</v>
+        <v>163</v>
       </c>
       <c r="C2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D2" t="s">
         <v>34</v>
-      </c>
-      <c r="D2" t="s">
-        <v>35</v>
       </c>
       <c r="E2">
         <v>5</v>
       </c>
       <c r="F2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="G2" t="s">
+        <v>88</v>
+      </c>
+      <c r="H2" t="s">
+        <v>98</v>
+      </c>
+      <c r="I2" t="s">
         <v>103</v>
       </c>
-      <c r="H2" t="s">
-        <v>113</v>
-      </c>
-      <c r="I2" t="s">
-        <v>118</v>
-      </c>
       <c r="J2" t="s">
-        <v>121</v>
+        <v>106</v>
       </c>
       <c r="K2" t="s">
-        <v>122</v>
+        <v>107</v>
       </c>
       <c r="L2" t="s">
-        <v>174</v>
-      </c>
-      <c r="M2" s="3">
+        <v>159</v>
+      </c>
+      <c r="M2" s="6">
         <v>45294</v>
       </c>
-      <c r="N2" s="4">
+      <c r="N2" s="3">
         <v>13000000</v>
       </c>
       <c r="O2" t="s">
-        <v>101</v>
-      </c>
-      <c r="P2" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C3" t="s">
         <v>51</v>
       </c>
-      <c r="C3" t="s">
-        <v>56</v>
-      </c>
       <c r="D3" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="E3">
         <v>2</v>
       </c>
       <c r="F3" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="G3" t="s">
-        <v>108</v>
+        <v>93</v>
       </c>
       <c r="H3" t="s">
-        <v>124</v>
+        <v>109</v>
       </c>
       <c r="I3" t="s">
-        <v>126</v>
+        <v>111</v>
       </c>
       <c r="J3" t="s">
-        <v>129</v>
+        <v>114</v>
       </c>
       <c r="K3" t="s">
-        <v>132</v>
+        <v>117</v>
       </c>
       <c r="L3" t="s">
-        <v>134</v>
-      </c>
-      <c r="M3" s="3">
+        <v>119</v>
+      </c>
+      <c r="M3" s="6">
         <v>45316</v>
       </c>
       <c r="N3">
         <v>12000000</v>
       </c>
       <c r="O3" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D4" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E4">
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="G4" t="s">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="H4" t="s">
-        <v>114</v>
+        <v>99</v>
       </c>
       <c r="I4" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="J4" t="s">
-        <v>121</v>
+        <v>106</v>
       </c>
       <c r="K4" t="s">
-        <v>122</v>
+        <v>107</v>
       </c>
       <c r="L4" t="s">
-        <v>175</v>
-      </c>
-      <c r="M4" s="3">
+        <v>160</v>
+      </c>
+      <c r="M4" s="6">
         <v>45325</v>
       </c>
       <c r="N4">
         <v>19000000</v>
       </c>
       <c r="O4" t="s">
-        <v>102</v>
-      </c>
-      <c r="P4" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="C5" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="D5" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="E5">
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="G5" t="s">
+        <v>97</v>
+      </c>
+      <c r="H5" t="s">
+        <v>109</v>
+      </c>
+      <c r="I5" t="s">
         <v>112</v>
       </c>
-      <c r="H5" t="s">
-        <v>124</v>
-      </c>
-      <c r="I5" t="s">
-        <v>127</v>
-      </c>
       <c r="J5" t="s">
-        <v>121</v>
+        <v>106</v>
       </c>
       <c r="K5" t="s">
-        <v>132</v>
+        <v>117</v>
       </c>
       <c r="L5" t="s">
-        <v>134</v>
-      </c>
-      <c r="M5" s="3">
+        <v>119</v>
+      </c>
+      <c r="M5" s="6">
         <v>45373</v>
       </c>
       <c r="N5">
         <v>20000000</v>
       </c>
       <c r="O5" t="s">
-        <v>102</v>
-      </c>
-      <c r="P5" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>179</v>
+        <v>164</v>
       </c>
       <c r="C6" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="D6" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E6">
         <v>5</v>
       </c>
       <c r="F6" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="G6" t="s">
+        <v>95</v>
+      </c>
+      <c r="H6" t="s">
         <v>110</v>
       </c>
-      <c r="H6" t="s">
-        <v>125</v>
-      </c>
       <c r="I6" t="s">
-        <v>128</v>
+        <v>113</v>
       </c>
       <c r="J6" t="s">
-        <v>129</v>
+        <v>114</v>
       </c>
       <c r="K6" t="s">
-        <v>133</v>
+        <v>118</v>
       </c>
       <c r="L6" t="s">
-        <v>135</v>
-      </c>
-      <c r="M6" s="3">
+        <v>120</v>
+      </c>
+      <c r="M6" s="6">
         <v>45399</v>
       </c>
       <c r="N6">
         <v>16000000</v>
       </c>
       <c r="O6" t="s">
-        <v>101</v>
-      </c>
-      <c r="P6" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>181</v>
+        <v>166</v>
       </c>
       <c r="C7" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D7" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E7">
         <v>2</v>
       </c>
       <c r="F7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G7" t="s">
-        <v>105</v>
+        <v>90</v>
       </c>
       <c r="H7" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
       <c r="I7" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="J7" t="s">
-        <v>121</v>
+        <v>106</v>
       </c>
       <c r="K7" t="s">
-        <v>123</v>
+        <v>108</v>
       </c>
       <c r="L7" t="s">
-        <v>176</v>
-      </c>
-      <c r="M7" s="3">
+        <v>161</v>
+      </c>
+      <c r="M7" s="6">
         <v>45415</v>
       </c>
       <c r="N7">
         <v>24000000</v>
       </c>
       <c r="O7" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>179</v>
+        <v>164</v>
       </c>
       <c r="C8" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="D8" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E8">
         <v>2</v>
       </c>
       <c r="F8" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="G8" t="s">
-        <v>111</v>
+        <v>96</v>
       </c>
       <c r="H8" t="s">
-        <v>125</v>
+        <v>110</v>
       </c>
       <c r="I8" t="s">
-        <v>128</v>
+        <v>113</v>
       </c>
       <c r="J8" t="s">
-        <v>130</v>
+        <v>115</v>
       </c>
       <c r="K8" t="s">
-        <v>133</v>
+        <v>118</v>
       </c>
       <c r="L8" t="s">
-        <v>135</v>
-      </c>
-      <c r="M8" s="3">
+        <v>120</v>
+      </c>
+      <c r="M8" s="6">
         <v>45427</v>
       </c>
       <c r="N8">
         <v>16000000</v>
       </c>
       <c r="O8" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C9" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="D9" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="E9">
         <v>3</v>
       </c>
       <c r="F9" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="G9" t="s">
-        <v>146</v>
+        <v>131</v>
       </c>
       <c r="H9" t="s">
-        <v>156</v>
+        <v>141</v>
       </c>
       <c r="I9" t="s">
-        <v>159</v>
+        <v>144</v>
       </c>
       <c r="J9" t="s">
-        <v>163</v>
+        <v>148</v>
       </c>
       <c r="K9" t="s">
-        <v>166</v>
+        <v>151</v>
       </c>
       <c r="L9" t="s">
-        <v>170</v>
-      </c>
-      <c r="M9" s="3">
+        <v>155</v>
+      </c>
+      <c r="M9" s="6">
         <v>45443</v>
       </c>
       <c r="N9">
         <v>180000</v>
       </c>
       <c r="O9" t="s">
-        <v>101</v>
-      </c>
-      <c r="P9" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B10" t="s">
-        <v>180</v>
+        <v>165</v>
       </c>
       <c r="C10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D10" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E10">
         <v>5</v>
       </c>
       <c r="F10" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="G10" t="s">
-        <v>106</v>
+        <v>91</v>
       </c>
       <c r="H10" t="s">
-        <v>116</v>
+        <v>101</v>
       </c>
       <c r="I10" t="s">
-        <v>119</v>
+        <v>104</v>
       </c>
       <c r="J10" t="s">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="K10" t="s">
-        <v>123</v>
+        <v>108</v>
       </c>
       <c r="L10" t="s">
-        <v>176</v>
-      </c>
-      <c r="M10" s="3">
+        <v>161</v>
+      </c>
+      <c r="M10" s="6">
         <v>45432</v>
       </c>
       <c r="N10">
         <v>35000000</v>
       </c>
       <c r="O10" t="s">
-        <v>101</v>
-      </c>
-      <c r="P10" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B11" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="C11" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="D11" t="s">
-        <v>48</v>
-      </c>
-      <c r="E11" s="5">
+        <v>44</v>
+      </c>
+      <c r="E11" s="4">
         <v>2</v>
       </c>
       <c r="F11" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="G11" t="s">
-        <v>147</v>
+        <v>132</v>
       </c>
       <c r="H11" t="s">
-        <v>157</v>
+        <v>142</v>
       </c>
       <c r="I11" t="s">
-        <v>160</v>
+        <v>145</v>
       </c>
       <c r="J11" t="s">
-        <v>159</v>
+        <v>144</v>
       </c>
       <c r="K11" t="s">
-        <v>167</v>
+        <v>152</v>
       </c>
       <c r="L11" t="s">
-        <v>170</v>
-      </c>
-      <c r="M11" s="3">
+        <v>155</v>
+      </c>
+      <c r="M11" s="6">
         <v>45444</v>
       </c>
       <c r="N11">
         <v>2900000</v>
       </c>
       <c r="O11" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B12" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="C12" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="D12" t="s">
-        <v>48</v>
-      </c>
-      <c r="E12" s="5">
+        <v>44</v>
+      </c>
+      <c r="E12" s="4">
         <v>2</v>
       </c>
       <c r="F12" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="G12" t="s">
-        <v>148</v>
+        <v>133</v>
       </c>
       <c r="H12" t="s">
-        <v>157</v>
+        <v>142</v>
       </c>
       <c r="I12" t="s">
-        <v>160</v>
+        <v>145</v>
       </c>
       <c r="J12" t="s">
-        <v>159</v>
+        <v>144</v>
       </c>
       <c r="K12" t="s">
-        <v>167</v>
+        <v>152</v>
       </c>
       <c r="L12" t="s">
-        <v>170</v>
-      </c>
-      <c r="M12" s="3">
+        <v>155</v>
+      </c>
+      <c r="M12" s="6">
         <v>45453</v>
       </c>
       <c r="N12">
         <v>2900000</v>
       </c>
       <c r="O12" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B13" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C13" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D13" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E13">
         <v>5</v>
       </c>
       <c r="F13" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="G13" t="s">
+        <v>92</v>
+      </c>
+      <c r="H13" t="s">
+        <v>102</v>
+      </c>
+      <c r="I13" t="s">
+        <v>103</v>
+      </c>
+      <c r="J13" t="s">
+        <v>106</v>
+      </c>
+      <c r="K13" t="s">
         <v>107</v>
       </c>
-      <c r="H13" t="s">
-        <v>117</v>
-      </c>
-      <c r="I13" t="s">
-        <v>118</v>
-      </c>
-      <c r="J13" t="s">
-        <v>121</v>
-      </c>
-      <c r="K13" t="s">
-        <v>122</v>
-      </c>
       <c r="L13" t="s">
-        <v>176</v>
-      </c>
-      <c r="M13" s="3">
+        <v>161</v>
+      </c>
+      <c r="M13" s="6">
         <v>45455</v>
       </c>
       <c r="N13">
         <v>21000000</v>
       </c>
       <c r="O13" t="s">
-        <v>101</v>
-      </c>
-      <c r="P13" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B14" t="s">
-        <v>182</v>
+        <v>167</v>
       </c>
       <c r="C14" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="D14" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E14">
         <v>3</v>
       </c>
       <c r="F14" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="G14" t="s">
-        <v>136</v>
+        <v>121</v>
       </c>
       <c r="H14" t="s">
-        <v>138</v>
+        <v>123</v>
       </c>
       <c r="I14" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="J14" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="K14" t="s">
-        <v>123</v>
+        <v>108</v>
       </c>
       <c r="L14" t="s">
-        <v>176</v>
-      </c>
-      <c r="M14" s="3">
+        <v>161</v>
+      </c>
+      <c r="M14" s="6">
         <v>45474</v>
       </c>
       <c r="N14">
         <v>14000000</v>
       </c>
       <c r="O14" t="s">
-        <v>102</v>
-      </c>
-      <c r="P14" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B15" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="C15" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="D15" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E15">
         <v>5</v>
       </c>
       <c r="F15" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="G15" t="s">
-        <v>149</v>
+        <v>134</v>
       </c>
       <c r="H15" t="s">
-        <v>157</v>
+        <v>142</v>
       </c>
       <c r="I15" t="s">
-        <v>160</v>
+        <v>145</v>
       </c>
       <c r="J15" t="s">
-        <v>159</v>
+        <v>144</v>
       </c>
       <c r="K15" t="s">
-        <v>167</v>
+        <v>152</v>
       </c>
       <c r="L15" t="s">
-        <v>170</v>
-      </c>
-      <c r="M15" s="3">
+        <v>155</v>
+      </c>
+      <c r="M15" s="6">
         <v>45483</v>
       </c>
       <c r="N15">
         <v>6100000</v>
       </c>
-      <c r="O15" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="P15" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="O15" s="4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B16" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C16" t="s">
-        <v>177</v>
+        <v>162</v>
       </c>
       <c r="D16" t="s">
-        <v>140</v>
+        <v>125</v>
       </c>
       <c r="E16">
         <v>2</v>
       </c>
       <c r="F16" t="s">
-        <v>141</v>
+        <v>126</v>
       </c>
       <c r="G16" t="s">
-        <v>137</v>
+        <v>122</v>
       </c>
       <c r="H16" t="s">
-        <v>139</v>
+        <v>124</v>
       </c>
       <c r="I16" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="J16" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="K16" t="s">
-        <v>122</v>
+        <v>107</v>
       </c>
       <c r="L16" t="s">
-        <v>142</v>
-      </c>
-      <c r="M16" s="3">
+        <v>127</v>
+      </c>
+      <c r="M16" s="6">
         <v>45514</v>
       </c>
       <c r="N16">
         <v>11000000</v>
       </c>
       <c r="O16" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B17" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C17" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="D17" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="E17">
         <v>5</v>
       </c>
       <c r="F17" t="s">
-        <v>143</v>
+        <v>128</v>
       </c>
       <c r="G17" t="s">
-        <v>150</v>
+        <v>135</v>
       </c>
       <c r="H17" t="s">
-        <v>156</v>
+        <v>141</v>
       </c>
       <c r="I17" t="s">
-        <v>159</v>
+        <v>144</v>
       </c>
       <c r="J17" t="s">
-        <v>163</v>
+        <v>148</v>
       </c>
       <c r="K17" t="s">
-        <v>166</v>
+        <v>151</v>
       </c>
       <c r="L17" t="s">
-        <v>170</v>
-      </c>
-      <c r="M17" s="3">
+        <v>155</v>
+      </c>
+      <c r="M17" s="6">
         <v>45563</v>
       </c>
       <c r="N17">
         <v>180000</v>
       </c>
-      <c r="O17" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="P17" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="O17" s="4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B18" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="C18" t="s">
-        <v>144</v>
+        <v>129</v>
       </c>
       <c r="D18" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="E18">
         <v>5</v>
       </c>
       <c r="F18" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="G18" t="s">
-        <v>172</v>
+        <v>157</v>
       </c>
       <c r="H18" t="s">
-        <v>158</v>
+        <v>143</v>
       </c>
       <c r="I18" t="s">
-        <v>126</v>
+        <v>111</v>
       </c>
       <c r="J18" t="s">
-        <v>164</v>
+        <v>149</v>
       </c>
       <c r="K18" t="s">
-        <v>168</v>
+        <v>153</v>
       </c>
       <c r="L18" t="s">
-        <v>171</v>
-      </c>
-      <c r="M18" s="3">
+        <v>156</v>
+      </c>
+      <c r="M18" s="6">
         <v>45584</v>
       </c>
       <c r="N18">
         <v>2250000</v>
       </c>
       <c r="O18" t="s">
-        <v>102</v>
-      </c>
-      <c r="P18" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B19" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="C19" t="s">
-        <v>144</v>
+        <v>129</v>
       </c>
       <c r="D19" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="E19">
         <v>5</v>
       </c>
       <c r="F19" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="G19" t="s">
-        <v>173</v>
+        <v>158</v>
       </c>
       <c r="H19" t="s">
-        <v>158</v>
+        <v>143</v>
       </c>
       <c r="I19" t="s">
-        <v>126</v>
+        <v>111</v>
       </c>
       <c r="J19" t="s">
-        <v>164</v>
+        <v>149</v>
       </c>
       <c r="K19" t="s">
-        <v>168</v>
+        <v>153</v>
       </c>
       <c r="L19" t="s">
-        <v>171</v>
-      </c>
-      <c r="M19" s="3">
+        <v>156</v>
+      </c>
+      <c r="M19" s="6">
         <v>45593</v>
       </c>
       <c r="N19">
         <v>2250000</v>
       </c>
-      <c r="O19" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="P19" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="O19" s="4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B20" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="C20" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="D20" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E20">
         <v>2</v>
       </c>
       <c r="F20" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="G20" t="s">
-        <v>151</v>
+        <v>136</v>
       </c>
       <c r="H20" t="s">
-        <v>157</v>
+        <v>142</v>
       </c>
       <c r="I20" t="s">
-        <v>160</v>
+        <v>145</v>
       </c>
       <c r="J20" t="s">
-        <v>159</v>
+        <v>144</v>
       </c>
       <c r="K20" t="s">
-        <v>167</v>
+        <v>152</v>
       </c>
       <c r="L20" t="s">
-        <v>170</v>
-      </c>
-      <c r="M20" s="3">
+        <v>155</v>
+      </c>
+      <c r="M20" s="6">
         <v>45606</v>
       </c>
       <c r="N20">
         <v>6100000</v>
       </c>
-      <c r="O20" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="O20" s="4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B21" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="C21" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="D21" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="E21">
         <v>5</v>
       </c>
       <c r="F21" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="G21" t="s">
+        <v>94</v>
+      </c>
+      <c r="H21" t="s">
         <v>109</v>
       </c>
-      <c r="H21" t="s">
-        <v>124</v>
-      </c>
       <c r="I21" t="s">
-        <v>127</v>
+        <v>112</v>
       </c>
       <c r="J21" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="K21" t="s">
-        <v>132</v>
+        <v>117</v>
       </c>
       <c r="L21" t="s">
-        <v>134</v>
-      </c>
-      <c r="M21" s="3">
+        <v>119</v>
+      </c>
+      <c r="M21" s="6">
         <v>45615</v>
       </c>
       <c r="N21">
         <v>25000000</v>
       </c>
-      <c r="O21" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="P21" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="O21" s="4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B22" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C22" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="D22" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E22">
         <v>2</v>
       </c>
       <c r="F22" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="G22" t="s">
-        <v>152</v>
+        <v>137</v>
       </c>
       <c r="H22" t="s">
-        <v>156</v>
+        <v>141</v>
       </c>
       <c r="I22" t="s">
-        <v>161</v>
+        <v>146</v>
       </c>
       <c r="J22" t="s">
-        <v>165</v>
+        <v>150</v>
       </c>
       <c r="K22" t="s">
-        <v>166</v>
+        <v>151</v>
       </c>
       <c r="L22" t="s">
-        <v>170</v>
-      </c>
-      <c r="M22" s="3">
+        <v>155</v>
+      </c>
+      <c r="M22" s="6">
         <v>45623</v>
       </c>
       <c r="N22">
         <v>120000</v>
       </c>
       <c r="O22" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B23" t="s">
-        <v>145</v>
+        <v>130</v>
       </c>
       <c r="C23" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="D23" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="E23">
         <v>4</v>
       </c>
       <c r="F23" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="G23" t="s">
-        <v>153</v>
+        <v>138</v>
       </c>
       <c r="H23" t="s">
-        <v>156</v>
+        <v>141</v>
       </c>
       <c r="I23" t="s">
-        <v>162</v>
+        <v>147</v>
       </c>
       <c r="J23" t="s">
-        <v>161</v>
+        <v>146</v>
       </c>
       <c r="K23" t="s">
-        <v>166</v>
+        <v>151</v>
       </c>
       <c r="L23" t="s">
-        <v>170</v>
-      </c>
-      <c r="M23" s="3">
+        <v>155</v>
+      </c>
+      <c r="M23" s="6">
         <v>45628</v>
       </c>
       <c r="N23">
         <v>1800000</v>
       </c>
-      <c r="O23" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="O23" s="4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B24" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="C24" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="D24" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="E24">
         <v>4</v>
       </c>
       <c r="F24" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="G24" t="s">
+        <v>139</v>
+      </c>
+      <c r="H24" t="s">
+        <v>141</v>
+      </c>
+      <c r="I24" t="s">
+        <v>146</v>
+      </c>
+      <c r="J24" t="s">
+        <v>150</v>
+      </c>
+      <c r="K24" t="s">
         <v>154</v>
       </c>
-      <c r="H24" t="s">
-        <v>156</v>
-      </c>
-      <c r="I24" t="s">
-        <v>161</v>
-      </c>
-      <c r="J24" t="s">
-        <v>165</v>
-      </c>
-      <c r="K24" t="s">
-        <v>169</v>
-      </c>
       <c r="L24" t="s">
-        <v>170</v>
-      </c>
-      <c r="M24" s="3">
+        <v>155</v>
+      </c>
+      <c r="M24" s="6">
         <v>45636</v>
       </c>
       <c r="N24">
         <v>150000</v>
       </c>
-      <c r="O24" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="O24" s="4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B25" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C25" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="D25" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="E25">
         <v>3</v>
       </c>
       <c r="F25" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="G25" t="s">
+        <v>140</v>
+      </c>
+      <c r="H25" t="s">
+        <v>141</v>
+      </c>
+      <c r="I25" t="s">
+        <v>144</v>
+      </c>
+      <c r="J25" t="s">
+        <v>148</v>
+      </c>
+      <c r="K25" t="s">
+        <v>151</v>
+      </c>
+      <c r="L25" t="s">
         <v>155</v>
       </c>
-      <c r="H25" t="s">
-        <v>156</v>
-      </c>
-      <c r="I25" t="s">
-        <v>159</v>
-      </c>
-      <c r="J25" t="s">
-        <v>163</v>
-      </c>
-      <c r="K25" t="s">
-        <v>166</v>
-      </c>
-      <c r="L25" t="s">
-        <v>170</v>
-      </c>
-      <c r="M25" s="3">
+      <c r="M25" s="6">
         <v>45638</v>
       </c>
       <c r="N25">
         <v>180000</v>
       </c>
       <c r="O25" t="s">
-        <v>102</v>
-      </c>
-      <c r="P25" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P25" xr:uid="{61CE36BB-B836-FE48-96B8-B2CA2E34C478}"/>
+  <autoFilter ref="A1:O25" xr:uid="{61CE36BB-B836-FE48-96B8-B2CA2E34C478}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>